<commit_message>
Add May 12 receipt entries
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R2f4a95a86e3c406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R73c7c933057548b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R5a06687460a44477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="Rc496b0e235714b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R41dcd6f0d0fa4afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R2c1c2f267cee4e8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1339,6 +1339,742 @@
         <x:v>/Users/tools/Downloads/IMG_8757.JPG</x:v>
       </x:c>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>R20260512-LETAO</x:v>
+      </x:c>
+      <x:c r="C23" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>15:51</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>ルタオ みどり店</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>厚焼金パンひとり</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>パン</x:v>
+      </x:c>
+      <x:c r="H23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I23" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="J23" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="K23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L23" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="M23" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="N23" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O23" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
+      <x:c r="Q23" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C24" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>明治ブルガリアヨーグルト</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>乳製品</x:v>
+      </x:c>
+      <x:c r="H24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I24" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="J24" t="n">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="K24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" t="n">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="M24" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="N24" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="P24" t="str">
+        <x:v>2個 x 単158円</x:v>
+      </x:c>
+      <x:c r="Q24" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C25" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>オクラ すり納豆S</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>納豆</x:v>
+      </x:c>
+      <x:c r="H25" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I25" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="J25" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="K25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M25" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="N25" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O25" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="P25" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
+      <x:c r="Q25" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C26" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>マウントレーニア</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>飲料</x:v>
+      </x:c>
+      <x:c r="H26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I26" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="J26" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="K26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M26" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="N26" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O26" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="P26" t="str"/>
+      <x:c r="Q26" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C27" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>ニップト カップキューブ</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>食品</x:v>
+      </x:c>
+      <x:c r="H27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I27" t="n">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="J27" t="n">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="K27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" t="n">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="M27" t="n">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="N27" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O27" t="str">
+        <x:v>低</x:v>
+      </x:c>
+      <x:c r="P27" t="str">
+        <x:v>商品名は判読不確実</x:v>
+      </x:c>
+      <x:c r="Q27" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C28" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>こだわるセロリーぶどう</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>野菜・果物</x:v>
+      </x:c>
+      <x:c r="H28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I28" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="J28" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="K28" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="M28" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="N28" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O28" t="str">
+        <x:v>低</x:v>
+      </x:c>
+      <x:c r="P28" t="str">
+        <x:v>商品名は判読不確実</x:v>
+      </x:c>
+      <x:c r="Q28" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C29" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>タカラ55 イチゴ</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>食品</x:v>
+      </x:c>
+      <x:c r="H29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I29" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="J29" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="K29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="M29" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="N29" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O29" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="P29" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
+      <x:c r="Q29" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C30" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>厚揚げがんばれ!野菜</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>惣菜・豆腐</x:v>
+      </x:c>
+      <x:c r="H30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I30" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="J30" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="K30" t="n">
+        <x:v>-34</x:v>
+      </x:c>
+      <x:c r="L30" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="M30" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="N30" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O30" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="P30" t="str">
+        <x:v>20%値引</x:v>
+      </x:c>
+      <x:c r="Q30" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C31" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>人参</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>野菜</x:v>
+      </x:c>
+      <x:c r="H31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I31" t="n">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="J31" t="n">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="K31" t="n">
+        <x:v>-80</x:v>
+      </x:c>
+      <x:c r="L31" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="M31" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="N31" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O31" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>30%値引</x:v>
+      </x:c>
+      <x:c r="Q31" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C32" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>梅田 造産ブチとうふ</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>豆腐</x:v>
+      </x:c>
+      <x:c r="H32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I32" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="J32" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="K32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="M32" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="N32" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O32" t="str">
+        <x:v>低</x:v>
+      </x:c>
+      <x:c r="P32" t="str">
+        <x:v>商品名は判読不確実</x:v>
+      </x:c>
+      <x:c r="Q32" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C33" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>COOPサクたまごせ</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>食品</x:v>
+      </x:c>
+      <x:c r="H33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I33" t="n">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="J33" t="n">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="K33" t="n">
+        <x:v>-161</x:v>
+      </x:c>
+      <x:c r="L33" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="M33" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="N33" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O33" t="str">
+        <x:v>低</x:v>
+      </x:c>
+      <x:c r="P33" t="str">
+        <x:v>50%値引。商品名は判読不確実</x:v>
+      </x:c>
+      <x:c r="Q33" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C34" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>とまと1個</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>野菜</x:v>
+      </x:c>
+      <x:c r="H34" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I34" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J34" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="K34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="M34" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="N34" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O34" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="P34" t="str"/>
+      <x:c r="Q34" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C35" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>エノキ小</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>野菜</x:v>
+      </x:c>
+      <x:c r="H35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I35" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J35" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="K35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="M35" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="N35" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O35" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="P35" t="str"/>
+      <x:c r="Q35" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="C36" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Aカコーラゼロ1</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>飲料</x:v>
+      </x:c>
+      <x:c r="H36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I36" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="J36" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="K36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L36" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="M36" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="N36" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="O36" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
+      <x:c r="Q36" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1362,7 +2098,7 @@
         <x:v>店舗</x:v>
       </x:c>
       <x:c r="E1" s="2" t="str">
-        <x:v>小計(税抜)</x:v>
+        <x:v>小計(税抜/税込混在)</x:v>
       </x:c>
       <x:c r="F1" s="2" t="str">
         <x:v>税率</x:v>
@@ -1421,7 +2157,7 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>レシート左。商品名の一部は印字どおりに近く記録。</x:v>
+        <x:v>商品名の一部は印字どおりに近く記録。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1456,7 +2192,7 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>レシート左。今川焼は50%値引後で実質単価を算出。</x:v>
+        <x:v>今川焼は50%値引後で実質単価を算出。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1491,39 +2227,109 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>レシート右。CARDNET控えは同じ購入のカード控えとして扱い、二重計上しない。</x:v>
+        <x:v>CARDNET控えは同じ購入のカード控えとして扱い、二重計上しない。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>R20260512-LETAO</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>15:51</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>ルタオ みどり店</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="F5" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="G5" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H5" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>JCB</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>商品名はレシート画像から読める範囲。内消費税28円。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>レシート枚数</x:v>
+        <x:v>R20260512-COOP</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>明細行数</x:v>
-      </x:c>
-      <x:c r="B7" t="n">
-        <x:v>21</x:v>
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>2201</x:v>
+      </x:c>
+      <x:c r="F6" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="G6" t="n">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="H6" t="n">
+        <x:v>2201</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>領収書。値引は読取可能範囲で反映。税込合計2,201円。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>支払合計(税込)</x:v>
+        <x:v>レシート枚数</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>9457</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>税抜小計合計</x:v>
+        <x:v>明細行数</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>8758</x:v>
+        <x:v>35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>支払合計(税込)</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>12046</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>小計合計</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>11347</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1546,7 +2352,7 @@
         <x:v>最安店舗</x:v>
       </x:c>
       <x:c r="D1" s="2" t="str">
-        <x:v>最安実質単価(税抜)</x:v>
+        <x:v>最安実質単価</x:v>
       </x:c>
       <x:c r="E1" s="2" t="str">
         <x:v>購入日</x:v>
@@ -1570,246 +2376,248 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>いちごジャム</x:v>
+        <x:v>Aカコーラゼロ1</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>ジャム</x:v>
+        <x:v>飲料</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>業務スーパー 小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>358</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E2" t="n">
-        <x:v>46152</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>R20260510-GYOMU</x:v>
-      </x:c>
-      <x:c r="G2" t="str"/>
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>オールレーズン</x:v>
+        <x:v>COOPサクたまごせ</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>菓子</x:v>
+        <x:v>食品</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>業務スーパー 小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>148</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E3" t="n">
-        <x:v>46152</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>R20260510-GYOMU</x:v>
-      </x:c>
-      <x:c r="G3" t="str"/>
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>50%値引。商品名は判読不確実</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>オレンジブレンド</x:v>
+        <x:v>いちごジャム</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>飲料</x:v>
+        <x:v>ジャム</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>業務スーパー 小樽店</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>198</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>46154</x:v>
+        <x:v>46152</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>R20260512-AEON</x:v>
+        <x:v>R20260510-GYOMU</x:v>
       </x:c>
       <x:c r="G4" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>じゃがいも バラ</x:v>
+        <x:v>エノキ小</x:v>
       </x:c>
       <x:c r="B5" t="str">
         <x:v>野菜</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E5" t="n">
         <x:v>46154</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>R20260512-AEON</x:v>
+        <x:v>R20260512-COOP</x:v>
       </x:c>
       <x:c r="G5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>ジャガイモキタアカリ</x:v>
+        <x:v>オールレーズン</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>野菜</x:v>
+        <x:v>菓子</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>業務スーパー 小樽店</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>298</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E6" t="n">
-        <x:v>46154</x:v>
+        <x:v>46152</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>R20260512-AEON</x:v>
+        <x:v>R20260510-GYOMU</x:v>
       </x:c>
       <x:c r="G6" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>ダブルソフト</x:v>
+        <x:v>オクラ すり納豆S</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>パン</x:v>
+        <x:v>納豆</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>180</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E7" t="n">
         <x:v>46154</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>R20260512-AEON</x:v>
-      </x:c>
-      <x:c r="G7" t="str"/>
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>マルちゃんみそ味ラーメン</x:v>
+        <x:v>オレンジブレンド</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>麺類</x:v>
+        <x:v>飲料</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D8" t="n">
-        <x:v>375</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="E8" t="n">
-        <x:v>46151</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>R20260509-AEON</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>3個 x 単375円</x:v>
-      </x:c>
+        <x:v>R20260512-AEON</x:v>
+      </x:c>
+      <x:c r="G8" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>メンタームのど飴</x:v>
+        <x:v>こだわるセロリーぶどう</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>菓子</x:v>
+        <x:v>野菜・果物</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D9" t="n">
-        <x:v>185</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E9" t="n">
         <x:v>46154</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>R20260512-AEON</x:v>
+        <x:v>R20260512-COOP</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>商品名は画像から読める範囲</x:v>
+        <x:v>商品名は判読不確実</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>愛別産イエスななつぼし</x:v>
+        <x:v>じゃがいも バラ</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>米</x:v>
+        <x:v>野菜</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D10" t="n">
-        <x:v>3584</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E10" t="n">
-        <x:v>46151</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>R20260509-AEON</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>5kg等の容量は画像から未確認</x:v>
-      </x:c>
+        <x:v>R20260512-AEON</x:v>
+      </x:c>
+      <x:c r="G10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>強炭酸水レモン</x:v>
+        <x:v>ジャガイモキタアカリ</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>飲料</x:v>
+        <x:v>野菜</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>業務スーパー 小樽店</x:v>
+        <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D11" t="n">
-        <x:v>38</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="E11" t="n">
-        <x:v>46152</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>R20260510-GYOMU</x:v>
+        <x:v>R20260512-AEON</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>今川焼(あまおう苺)</x:v>
+        <x:v>タカラ55 イチゴ</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>菓子</x:v>
+        <x:v>食品</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D12" t="n">
-        <x:v>164</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E12" t="n">
         <x:v>46154</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>R20260512-AEON</x:v>
+        <x:v>R20260512-COOP</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>50%値引</x:v>
+        <x:v>商品名は画像から読める範囲</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>山崎スイートバターB5</x:v>
+        <x:v>ダブルソフト</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>パン</x:v>
@@ -1818,93 +2626,93 @@
         <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D13" t="n">
-        <x:v>100</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="E13" t="n">
-        <x:v>46151</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>R20260509-AEON</x:v>
+        <x:v>R20260512-AEON</x:v>
       </x:c>
       <x:c r="G13" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>松屋 生沖縄黒飴</x:v>
+        <x:v>とまと1個</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>菓子</x:v>
+        <x:v>野菜</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D14" t="n">
-        <x:v>185</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E14" t="n">
         <x:v>46154</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>R20260512-AEON</x:v>
+        <x:v>R20260512-COOP</x:v>
       </x:c>
       <x:c r="G14" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>生くろわっさん</x:v>
+        <x:v>ニップト カップキューブ</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>パン</x:v>
+        <x:v>食品</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D15" t="n">
-        <x:v>120</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="E15" t="n">
-        <x:v>46151</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>R20260509-AEON</x:v>
-      </x:c>
-      <x:c r="G15" t="str"/>
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>商品名は判読不確実</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>生ます</x:v>
+        <x:v>マウントレーニア</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>魚介</x:v>
+        <x:v>飲料</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D16" t="n">
-        <x:v>241</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E16" t="n">
-        <x:v>46151</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>R20260509-AEON</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>50%値引</x:v>
-      </x:c>
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G16" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>生乳プレーンヨーグルト</x:v>
+        <x:v>マルちゃんみそ味ラーメン</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>乳製品</x:v>
+        <x:v>麺類</x:v>
       </x:c>
       <x:c r="C17" t="str">
         <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D17" t="n">
-        <x:v>198</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="E17" t="n">
         <x:v>46151</x:v>
@@ -1912,41 +2720,45 @@
       <x:c r="F17" t="str">
         <x:v>R20260509-AEON</x:v>
       </x:c>
-      <x:c r="G17" t="str"/>
+      <x:c r="G17" t="str">
+        <x:v>3個 x 単375円</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>雪印 北海道バター</x:v>
+        <x:v>メンタームのど飴</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>乳製品</x:v>
+        <x:v>菓子</x:v>
       </x:c>
       <x:c r="C18" t="str">
         <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D18" t="n">
-        <x:v>398</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E18" t="n">
-        <x:v>46151</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F18" t="str">
-        <x:v>R20260509-AEON</x:v>
-      </x:c>
-      <x:c r="G18" t="str"/>
+        <x:v>R20260512-AEON</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>東ハトふんわり4連</x:v>
+        <x:v>愛別産イエスななつぼし</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>菓子</x:v>
+        <x:v>米</x:v>
       </x:c>
       <x:c r="C19" t="str">
         <x:v>イオン小樽店</x:v>
       </x:c>
       <x:c r="D19" t="n">
-        <x:v>148</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E19" t="n">
         <x:v>46151</x:v>
@@ -1955,21 +2767,21 @@
         <x:v>R20260509-AEON</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>商品名は画像から読める範囲</x:v>
+        <x:v>5kg等の容量は画像から未確認</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>粉末黒糖</x:v>
+        <x:v>強炭酸水レモン</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>砂糖・甘味料</x:v>
+        <x:v>飲料</x:v>
       </x:c>
       <x:c r="C20" t="str">
         <x:v>業務スーパー 小樽店</x:v>
       </x:c>
       <x:c r="D20" t="n">
-        <x:v>548</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E20" t="n">
         <x:v>46152</x:v>
@@ -1981,24 +2793,334 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
+        <x:v>厚焼金パンひとり</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>パン</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>ルタオ みどり店</x:v>
+      </x:c>
+      <x:c r="D21" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="E21" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>R20260512-LETAO</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>厚揚げがんばれ!野菜</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>惣菜・豆腐</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="D22" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="E22" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>20%値引</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>今川焼(あまおう苺)</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>菓子</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D23" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="E23" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>R20260512-AEON</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>50%値引</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>山崎スイートバターB5</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>パン</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E24" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G24" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>松屋 生沖縄黒飴</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>菓子</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D25" t="n">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="E25" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>R20260512-AEON</x:v>
+      </x:c>
+      <x:c r="G25" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>人参</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>野菜</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="D26" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="E26" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>30%値引</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>生くろわっさん</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>パン</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D27" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="E27" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G27" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>生ます</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>魚介</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D28" t="n">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="E28" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>50%値引</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>生乳プレーンヨーグルト</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>乳製品</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D29" t="n">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="E29" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G29" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>雪印 北海道バター</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>乳製品</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D30" t="n">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="E30" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G30" t="str"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>東ハトふんわり4連</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>菓子</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D31" t="n">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="E31" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>商品名は画像から読める範囲</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>梅田 造産ブチとうふ</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>豆腐</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="D32" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="E32" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>商品名は判読不確実</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>粉末黒糖</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>砂糖・甘味料</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>業務スーパー 小樽店</x:v>
+      </x:c>
+      <x:c r="D33" t="n">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="E33" t="n">
+        <x:v>46152</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>R20260510-GYOMU</x:v>
+      </x:c>
+      <x:c r="G33" t="str"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
         <x:v>北海道サツラク牛乳</x:v>
       </x:c>
-      <x:c r="B21" t="str">
+      <x:c r="B34" t="str">
         <x:v>乳製品</x:v>
       </x:c>
-      <x:c r="C21" t="str">
-        <x:v>イオン小樽店</x:v>
-      </x:c>
-      <x:c r="D21" t="n">
+      <x:c r="C34" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D34" t="n">
         <x:v>238</x:v>
       </x:c>
-      <x:c r="E21" t="n">
+      <x:c r="E34" t="n">
         <x:v>46151</x:v>
       </x:c>
-      <x:c r="F21" t="str">
+      <x:c r="F34" t="str">
         <x:v>R20260509-AEON</x:v>
       </x:c>
-      <x:c r="G21" t="str"/>
+      <x:c r="G34" t="str"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>明治ブルガリアヨーグルト</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>乳製品</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="D35" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="E35" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>2個 x 単158円</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add April fuel receipt entry
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="Rc496b0e235714b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R41dcd6f0d0fa4afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R2c1c2f267cee4e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="Rd5ce3d6abce742d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R42b54cb5567a4169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="Rdb0d447d36474edd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2075,6 +2075,59 @@
         <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
       </x:c>
     </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>R20260412-APOLLO</x:v>
+      </x:c>
+      <x:c r="C37" t="n">
+        <x:v>46124</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>13:05</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>apollostation 北海道エネルギー 小樽市内店</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>灯油</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>燃料</x:v>
+      </x:c>
+      <x:c r="H37" t="n">
+        <x:v>41.96</x:v>
+      </x:c>
+      <x:c r="I37" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="J37" t="n">
+        <x:v>6042.24</x:v>
+      </x:c>
+      <x:c r="K37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" t="n">
+        <x:v>6042.24</x:v>
+      </x:c>
+      <x:c r="M37" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="N37" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O37" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
+        <x:v>41.96L x 単価144円</x:v>
+      </x:c>
+      <x:c r="Q37" t="str">
+        <x:v>/Users/tools/Downloads/IMG_8761 2.JPG</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2300,12 +2353,47 @@
         <x:v>領収書。値引は読取可能範囲で反映。税込合計2,201円。</x:v>
       </x:c>
     </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>R20260412-APOLLO</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
+        <x:v>46124</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>13:05</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>apollostation 北海道エネルギー 小樽市内店</x:v>
+      </x:c>
+      <x:c r="E7" t="n">
+        <x:v>6042</x:v>
+      </x:c>
+      <x:c r="F7" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G7" t="n">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="H7" t="n">
+        <x:v>6042</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>灯油 41.96L、単価144円。内税10%対象。</x:v>
+      </x:c>
+    </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
         <x:v>レシート枚数</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2313,7 +2401,7 @@
         <x:v>明細行数</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2321,7 +2409,7 @@
         <x:v>支払合計(税込)</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>12046</x:v>
+        <x:v>18088</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2329,7 +2417,7 @@
         <x:v>小計合計</x:v>
       </x:c>
       <x:c r="B11" t="n">
-        <x:v>11347</x:v>
+        <x:v>17389</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3036,89 +3124,112 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
-        <x:v>梅田 造産ブチとうふ</x:v>
+        <x:v>灯油</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>豆腐</x:v>
+        <x:v>燃料</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>COOP SAPPORO みどり店</x:v>
+        <x:v>apollostation 北海道エネルギー 小樽市内店</x:v>
       </x:c>
       <x:c r="D32" t="n">
-        <x:v>450</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="E32" t="n">
-        <x:v>46154</x:v>
+        <x:v>46124</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>R20260512-COOP</x:v>
+        <x:v>R20260412-APOLLO</x:v>
       </x:c>
       <x:c r="G32" t="str">
-        <x:v>商品名は判読不確実</x:v>
+        <x:v>41.96L x 単価144円</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>粉末黒糖</x:v>
+        <x:v>梅田 造産ブチとうふ</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>砂糖・甘味料</x:v>
+        <x:v>豆腐</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>業務スーパー 小樽店</x:v>
+        <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D33" t="n">
-        <x:v>548</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="E33" t="n">
-        <x:v>46152</x:v>
+        <x:v>46154</x:v>
       </x:c>
       <x:c r="F33" t="str">
-        <x:v>R20260510-GYOMU</x:v>
-      </x:c>
-      <x:c r="G33" t="str"/>
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>商品名は判読不確実</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>北海道サツラク牛乳</x:v>
+        <x:v>粉末黒糖</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>乳製品</x:v>
+        <x:v>砂糖・甘味料</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>イオン小樽店</x:v>
+        <x:v>業務スーパー 小樽店</x:v>
       </x:c>
       <x:c r="D34" t="n">
-        <x:v>238</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="E34" t="n">
-        <x:v>46151</x:v>
+        <x:v>46152</x:v>
       </x:c>
       <x:c r="F34" t="str">
-        <x:v>R20260509-AEON</x:v>
+        <x:v>R20260510-GYOMU</x:v>
       </x:c>
       <x:c r="G34" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>明治ブルガリアヨーグルト</x:v>
+        <x:v>北海道サツラク牛乳</x:v>
       </x:c>
       <x:c r="B35" t="str">
         <x:v>乳製品</x:v>
       </x:c>
       <x:c r="C35" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="D35" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="E35" t="n">
+        <x:v>46151</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="G35" t="str"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>明治ブルガリアヨーグルト</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>乳製品</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
         <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
-      <x:c r="D35" t="n">
+      <x:c r="D36" t="n">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="E35" t="n">
-        <x:v>46154</x:v>
-      </x:c>
-      <x:c r="F35" t="str">
+      <x:c r="E36" t="n">
+        <x:v>46154</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
         <x:v>R20260512-COOP</x:v>
       </x:c>
-      <x:c r="G35" t="str">
+      <x:c r="G36" t="str">
         <x:v>2個 x 単158円</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Store receipt images with ledger
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="Rd5ce3d6abce742d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R42b54cb5567a4169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="Rdb0d447d36474edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R7aa439c75eb444be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="Rf50c1003f72f43b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R9ae8147de4534856"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2171,7 +2171,9 @@
       <x:c r="K1" s="2" t="str">
         <x:v>備考</x:v>
       </x:c>
-      <x:c r="L1" s="2"/>
+      <x:c r="L1" s="2" t="str">
+        <x:v>画像</x:v>
+      </x:c>
       <x:c r="M1" s="2"/>
       <x:c r="N1" s="2"/>
       <x:c r="O1" s="2"/>
@@ -2212,6 +2214,9 @@
       <x:c r="K2" t="str">
         <x:v>商品名の一部は印字どおりに近く記録。</x:v>
       </x:c>
+      <x:c r="L2" t="str">
+        <x:v>receipt_images/R20260509-AEON_IMG_8759.JPG</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -2247,6 +2252,9 @@
       <x:c r="K3" t="str">
         <x:v>今川焼は50%値引後で実質単価を算出。</x:v>
       </x:c>
+      <x:c r="L3" t="str">
+        <x:v>receipt_images/R20260512-AEON_IMG_8757.JPG</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -2282,6 +2290,9 @@
       <x:c r="K4" t="str">
         <x:v>CARDNET控えは同じ購入のカード控えとして扱い、二重計上しない。</x:v>
       </x:c>
+      <x:c r="L4" t="str">
+        <x:v>receipt_images/R20260510-GYOMU_IMG_8757.JPG</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -2317,6 +2328,9 @@
       <x:c r="K5" t="str">
         <x:v>商品名はレシート画像から読める範囲。内消費税28円。</x:v>
       </x:c>
+      <x:c r="L5" t="str">
+        <x:v>receipt_images/R20260512-LETAO_IMG_8760.JPG</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
@@ -2352,6 +2366,9 @@
       <x:c r="K6" t="str">
         <x:v>領収書。値引は読取可能範囲で反映。税込合計2,201円。</x:v>
       </x:c>
+      <x:c r="L6" t="str">
+        <x:v>receipt_images/R20260512-COOP_IMG_8760.JPG</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -2387,36 +2404,39 @@
       <x:c r="K7" t="str">
         <x:v>灯油 41.96L、単価144円。内税10%対象。</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>レシート枚数</x:v>
-      </x:c>
-      <x:c r="B8" t="n">
-        <x:v>6</x:v>
+      <x:c r="L7" t="str">
+        <x:v>receipt_images/R20260412-APOLLO_IMG_8761_2.JPG</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>明細行数</x:v>
+        <x:v>レシート枚数</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>36</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>支払合計(税込)</x:v>
+        <x:v>明細行数</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>18088</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
+        <x:v>支払合計(税込)</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>18088</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
         <x:v>小計合計</x:v>
       </x:c>
-      <x:c r="B11" t="n">
+      <x:c r="B12" t="n">
         <x:v>17389</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Correct tofu receipt entry
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R7aa439c75eb444be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="Rf50c1003f72f43b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R9ae8147de4534856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R8fe41fa5f2ea4bb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R206907cf7be4404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R043d7c1295234aaf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1831,7 +1831,7 @@
         <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>梅田 造産ブチとうふ</x:v>
+        <x:v>菊田堂さんとうふ</x:v>
       </x:c>
       <x:c r="G32" t="str">
         <x:v>豆腐</x:v>
@@ -1840,28 +1840,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I32" t="n">
-        <x:v>450</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J32" t="n">
-        <x:v>450</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L32" t="n">
-        <x:v>450</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M32" t="n">
-        <x:v>450</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="N32" t="n">
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>低</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="P32" t="str">
-        <x:v>商品名は判読不確実</x:v>
+        <x:v>150円に訂正</x:v>
       </x:c>
       <x:c r="Q32" t="str">
         <x:v>/Users/tools/Downloads/IMG_8760.JPG</x:v>
@@ -3167,7 +3167,7 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>梅田 造産ブチとうふ</x:v>
+        <x:v>菊田堂さんとうふ</x:v>
       </x:c>
       <x:c r="B33" t="str">
         <x:v>豆腐</x:v>
@@ -3176,7 +3176,7 @@
         <x:v>COOP SAPPORO みどり店</x:v>
       </x:c>
       <x:c r="D33" t="n">
-        <x:v>450</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E33" t="n">
         <x:v>46154</x:v>
@@ -3185,7 +3185,7 @@
         <x:v>R20260512-COOP</x:v>
       </x:c>
       <x:c r="G33" t="str">
-        <x:v>商品名は判読不確実</x:v>
+        <x:v>150円に訂正</x:v>
       </x:c>
     </x:row>
     <x:row r="34">

</xml_diff>

<commit_message>
Resolve Gyomu receipt reconciliation
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -288,7 +288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q133"/>
+  <dimension ref="A1:Q135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8246,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8374,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8438,7 +8438,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8502,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8566,7 +8566,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8704,7 +8704,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8773,7 +8773,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8906,7 +8906,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -8970,7 +8970,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -9034,7 +9034,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -9232,6 +9232,144 @@
       <c r="Q133" t="inlineStr">
         <is>
           <t>receipt_images/R20260423-DCM-1619_IMG_8763_2.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>R20260423-GYOMU-1651</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>業務スーパー 小樽店</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>ラガシュ クリーミー豆</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>食品</t>
+        </is>
+      </c>
+      <c r="H134" t="n">
+        <v>1</v>
+      </c>
+      <c r="I134" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="J134" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="K134" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L134" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="M134" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>IMG_8766で追加。商品名は読める範囲</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>R20260423-GYOMU-1651</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>業務スーパー 小樽店</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>TSコーヒーフィルター2-4杯用</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>日用品</t>
+        </is>
+      </c>
+      <c r="H135" t="n">
+        <v>1</v>
+      </c>
+      <c r="I135" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="J135" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="K135" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L135" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="M135" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="N135" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>IMG_8766で追加</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -10200,12 +10338,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>明細読取に差額あり（897円）。画像の一部が不鮮明。</t>
+          <t>IMG_8766で再確認。明細合計一致。</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>receipt_images/R20260423-GYOMU-1651_IMG_8763_2.JPG</t>
+          <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
         </is>
       </c>
     </row>
@@ -10339,7 +10477,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -10382,7 +10520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -10450,7 +10588,7 @@
       <c r="D2" s="5" t="n">
         <v>161</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="8" t="n">
         <v>46154</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -10544,7 +10682,7 @@
       <c r="D5" s="5" t="n">
         <v>161</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="8" t="n">
         <v>46154</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -10622,73 +10760,78 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TVバナナ</t>
+          <t>TSコーヒーフィルター2-4杯用</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>日用品</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>46152</v>
+        <v>46135</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2個 x 単70円</t>
+          <t>IMG_8766で追加</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>いちごジャム</t>
+          <t>TVバナナ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ジャム</t>
+          <t>果物</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>358</v>
-      </c>
-      <c r="E9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E9" s="8" t="n">
         <v>46152</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>R20260510-GYOMU</t>
+          <t>R20260510-AEON-1911</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2個 x 単70円</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>おぷうさんカレー クラウン5枚</t>
+          <t>いちごジャム</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>食品</t>
+          <t>ジャム</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -10697,120 +10840,120 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>125</v>
+        <v>358</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46135</v>
+        <v>46152</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>商品名は判読不確実</t>
+          <t>R20260510-GYOMU</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>かれい</t>
+          <t>おぷうさんカレー クラウン5枚</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>食品</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>303</v>
+        <v>125</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46146</v>
+        <v>46135</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>こだわるセロリーぶどう</t>
+          <t>かれい</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>野菜・果物</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>215</v>
-      </c>
-      <c r="E12" t="n">
-        <v>46154</v>
+        <v>303</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46146</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>商品名は判読不確実</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>じゃがいも</t>
+          <t>こだわるセロリーぶどう</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>野菜・果物</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>298</v>
+        <v>215</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>46135</v>
+        <v>46154</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260512-COOP</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>じゃがいも バラ</t>
+          <t>じゃがいも</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -10824,26 +10967,26 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="E14" t="n">
-        <v>46154</v>
+        <v>298</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>その他惣つま貝</t>
+          <t>じゃがいも バラ</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -10852,26 +10995,21 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>215</v>
+        <v>45</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>50%値引。商品名は判読不確実</t>
+          <t>R20260512-AEON</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>その他惣菜つま貝</t>
+          <t>その他惣つま貝</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -10885,14 +11023,14 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>236</v>
+        <v>215</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>46147</v>
+        <v>46146</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -10904,12 +11042,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>たい焼き</t>
+          <t>その他惣菜つま貝</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -10918,153 +11056,158 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>124</v>
+        <v>236</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>50%値引。商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>とまと1個</t>
+          <t>たい焼き</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="E18" t="n">
-        <v>46154</v>
+        <v>124</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>46139</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>にぎり鮨盛り</t>
+          <t>とまと1個</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>990</v>
+        <v>50</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>46147</v>
+        <v>46154</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260512-COOP</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ぷどうゼリー</t>
+          <t>にぎり鮨盛り</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>寿司</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>イオン マックスバリュ手宮店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>98</v>
+        <v>990</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>46141</v>
+        <v>46147</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>R20260429-AEON-MAXVALU-1437</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>商品名は画像から読める範囲</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>もっちり仕込み食パン</t>
+          <t>ぷどうゼリー</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>イオン マックスバリュ手宮店</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>46146</v>
+        <v>46141</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260429-AEON-MAXVALU-1437</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>もっちり焦しキャラメル</t>
+          <t>もっちり仕込み食パン</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -11073,7 +11216,7 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="E22" s="8" t="n">
         <v>46146</v>
@@ -11083,110 +11226,105 @@
           <t>R20260504-AEON-1918</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>50%値引</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>もみがらくん炭50L</t>
+          <t>もっちり焦しキャラメル</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>園芸</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DCM 手宮店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1408</v>
+        <v>79</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>46135</v>
+        <v>46146</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>R20260423-DCM-1619</t>
+          <t>R20260504-AEON-1918</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>アップルサラダ900</t>
+          <t>もみがらくん炭50L</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>園芸</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>DCM 手宮店</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>208</v>
+        <v>1408</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>46139</v>
+        <v>46135</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>2個 x 単298円、30%値引</t>
+          <t>R20260423-DCM-1619</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>アンパンマン パン ビーゼ</t>
+          <t>アップルサラダ900</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>イオン マックスバリュ手宮店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>128</v>
+        <v>208</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>46141</v>
+        <v>46139</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>R20260429-AEON-MAXVALU-1437</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>商品名は画像から読める範囲</t>
+          <t>2個 x 単298円、30%値引</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>アンパンマンのパンケーキ</t>
+          <t>アンパンマン パン ビーゼ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -11196,25 +11334,30 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>イオン マックスバリュ手宮店</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>46141</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>R20260429-AEON-1746</t>
+          <t>R20260429-AEON-MAXVALU-1437</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>アンパンマンのミニスナ</t>
+          <t>アンパンマンのパンケーキ</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -11224,96 +11367,96 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>イオン マックスバリュ手宮店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>151</v>
+        <v>120</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>46141</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>R20260429-AEON-MAXVALU-1437</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>10%値引</t>
+          <t>R20260429-AEON-1746</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>イタリアンプリネス</t>
+          <t>アンパンマンのミニスナ</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>食品</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン マックスバリュ手宮店</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>298</v>
+        <v>151</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>46135</v>
+        <v>46141</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260429-AEON-MAXVALU-1437</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>商品名は判読不確実</t>
+          <t>10%値引</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>エノキ小</t>
+          <t>イタリアンプリネス</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>食品</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="E29" t="n">
-        <v>46154</v>
+        <v>298</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260423-GYOMU-1651</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>オクラ すり納豆S</t>
+          <t>エノキ小</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>納豆</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -11322,59 +11465,59 @@
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="E30" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" s="8" t="n">
         <v>46154</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>R20260512-COOP</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>オレンジブレンド</t>
+          <t>オクラ すり納豆S</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>飲料</t>
+          <t>納豆</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>198</v>
-      </c>
-      <c r="E31" t="n">
+        <v>150</v>
+      </c>
+      <c r="E31" s="8" t="n">
         <v>46154</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
+          <t>R20260512-COOP</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>オールドファッションチョコ</t>
+          <t>オレンジブレンド</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>飲料</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -11383,26 +11526,21 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>79</v>
+        <v>198</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260512-AEON</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>オールレーズン</t>
+          <t>オールドファッションチョコ</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -11412,180 +11550,180 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>148</v>
-      </c>
-      <c r="E33" t="n">
-        <v>46152</v>
+        <v>79</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>46146</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>R20260510-GYOMU</t>
+          <t>R20260504-AEON-1918</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>カナダドライジンジャー</t>
+          <t>オールレーズン</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>飲料</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>98</v>
+        <v>148</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>46146</v>
+        <v>46152</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260510-GYOMU</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>カンロ 健康のど飴梅</t>
+          <t>カナダドライジンジャー</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>飲料</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>サンドラッグ 小樽稲穂店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>235</v>
+        <v>98</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>46152</v>
+        <v>46146</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>R20260510-SUNDRUG-1326</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>キングメロン ハーフ</t>
+          <t>カンロ 健康のど飴梅</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>サンドラッグ 小樽稲穂店</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>46135</v>
+        <v>46152</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260510-SUNDRUG-1326</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>グリーンもやし</t>
+          <t>キングメロン ハーフ</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>果物</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>29</v>
+        <v>249</v>
       </c>
       <c r="E37" s="8" t="n">
         <v>46135</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260423-AEON-1917</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>サンキ弁当</t>
+          <t>グリーンもやし</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>弁当</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>249</v>
+        <v>29</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>46147</v>
+        <v>46135</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>サーモン寿司小セット大</t>
+          <t>サンキ弁当</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>弁当</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -11594,14 +11732,14 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>349</v>
+        <v>249</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -11613,12 +11751,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ジャガイモキタアカリ</t>
+          <t>サーモン寿司小セット大</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>寿司</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -11627,92 +11765,92 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>298</v>
-      </c>
-      <c r="E40" t="n">
-        <v>46154</v>
+        <v>349</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>46139</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>タカラ55 イチゴ</t>
+          <t>ジャガイモキタアカリ</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>食品</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>215</v>
-      </c>
-      <c r="E41" t="n">
+        <v>298</v>
+      </c>
+      <c r="E41" s="8" t="n">
         <v>46154</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>商品名は画像から読める範囲</t>
+          <t>R20260512-AEON</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>タルタルチキン南蛮バー</t>
+          <t>タカラ55 イチゴ</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>食品</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>149</v>
+        <v>215</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>46139</v>
+        <v>46154</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260512-COOP</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ダブルソフト</t>
+          <t>タルタルチキン南蛮バー</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -11721,26 +11859,31 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>180</v>
-      </c>
-      <c r="E43" t="n">
-        <v>46154</v>
+        <v>149</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>46139</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>チキンカツカレー</t>
+          <t>ダブルソフト</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>弁当</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -11749,148 +11892,148 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>249</v>
+        <v>180</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260512-AEON</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ディルピクルス(ホール)</t>
+          <t>チキンカツカレー</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>食品</t>
+          <t>弁当</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>318</v>
+        <v>249</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>46135</v>
+        <v>46146</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260504-AEON-1918</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>トリニク</t>
+          <t>ディルピクルス(ホール)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>肉</t>
+          <t>食品</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>136</v>
+        <v>318</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>46146</v>
+        <v>46135</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ニップト カップキューブ</t>
+          <t>トリニク</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>食品</t>
+          <t>肉</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>257</v>
-      </c>
-      <c r="E47" t="n">
-        <v>46154</v>
+        <v>136</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>46146</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>商品名は判読不確実</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ハニーパイン</t>
+          <t>ニップト カップキューブ</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>食品</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>298</v>
+        <v>257</v>
       </c>
       <c r="E48" s="8" t="n">
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260512-COOP</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>バナナ</t>
+          <t>ハニーパイン</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -11904,26 +12047,26 @@
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>158</v>
+        <v>298</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>46147</v>
+        <v>46146</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ピーマン</t>
+          <t>バナナ</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>果物</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -11932,26 +12075,26 @@
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>98</v>
+        <v>158</v>
       </c>
       <c r="E50" s="8" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>フルーツフェスタ アップル</t>
+          <t>ピーマン</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>飲料</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -11960,26 +12103,21 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>196</v>
+        <v>98</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>46141</v>
+        <v>46146</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>R20260429-AEON-1746</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>10%値引</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>フルーツフェスタグレー</t>
+          <t>フルーツフェスタ アップル</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -11989,35 +12127,35 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>152</v>
+        <v>196</v>
       </c>
       <c r="E52" s="8" t="n">
-        <v>46135</v>
+        <v>46141</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260429-AEON-1746</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>30%値引</t>
+          <t>10%値引</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ベストバラエティ</t>
+          <t>フルーツフェスタグレー</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>飲料</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -12026,7 +12164,7 @@
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>268</v>
+        <v>152</v>
       </c>
       <c r="E53" s="8" t="n">
         <v>46135</v>
@@ -12036,49 +12174,49 @@
           <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>30%値引</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ホッケレイ</t>
+          <t>ベストバラエティ</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>157</v>
+        <v>268</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>46139</v>
+        <v>46135</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ホテル仕込み食パン</t>
+          <t>ホッケレイ</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -12087,26 +12225,31 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>288</v>
+        <v>157</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>46146</v>
+        <v>46139</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ホンカレイ</t>
+          <t>ホテル仕込み食パン</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -12115,64 +12258,59 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>141</v>
+        <v>288</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ボルシチ仕込みホット無糖</t>
+          <t>ホンカレイ</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>飲料</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>228</v>
+        <v>141</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>商品名は判読不確実</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ポテトチップス サワークリーム</t>
+          <t>ボルシチ仕込みホット無糖</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>飲料</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -12181,7 +12319,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>168</v>
+        <v>228</v>
       </c>
       <c r="E58" s="8" t="n">
         <v>46135</v>
@@ -12191,100 +12329,105 @@
           <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>商品名は判読不確実</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>マウントレーニア</t>
+          <t>ポテトチップス サワークリーム</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>飲料</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="E59" t="n">
-        <v>46154</v>
+        <v>168</v>
+      </c>
+      <c r="E59" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>マルちゃんみそ味ラーメン</t>
+          <t>マウントレーニア</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>麺類</t>
+          <t>飲料</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D60" s="5" t="n">
-        <v>375</v>
-      </c>
-      <c r="E60" t="n">
-        <v>46151</v>
+        <v>150</v>
+      </c>
+      <c r="E60" s="8" t="n">
+        <v>46154</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>3個 x 単375円</t>
+          <t>R20260512-COOP</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ミックスナッツ</t>
+          <t>マルちゃんみそ味ラーメン</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>麺類</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D61" s="5" t="n">
-        <v>438</v>
+        <v>375</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>46135</v>
+        <v>46151</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260509-AEON</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>3個 x 単375円</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ミルク風味グレーズクリ</t>
+          <t>ミックスナッツ</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -12294,35 +12437,30 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D62" s="5" t="n">
-        <v>79</v>
+        <v>438</v>
       </c>
       <c r="E62" s="8" t="n">
-        <v>46146</v>
+        <v>46135</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>50%値引。商品名は判読不確実</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>メロンカット</t>
+          <t>ミルク風味グレーズクリ</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -12331,31 +12469,31 @@
         </is>
       </c>
       <c r="D63" s="5" t="n">
-        <v>149</v>
+        <v>79</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>46152</v>
+        <v>46146</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>50%値引。商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>メンタームのど飴</t>
+          <t>メロンカット</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>果物</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -12364,26 +12502,26 @@
         </is>
       </c>
       <c r="D64" s="5" t="n">
-        <v>185</v>
-      </c>
-      <c r="E64" t="n">
-        <v>46154</v>
+        <v>149</v>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>46152</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
+          <t>R20260510-AEON-1911</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>商品名は画像から読める範囲</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>リスカ うまい輪チーズ</t>
+          <t>メンタームのど飴</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -12393,58 +12531,63 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D65" s="5" t="n">
-        <v>88</v>
+        <v>185</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>46135</v>
+        <v>46154</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260512-AEON</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>レギュラーガソリン</t>
+          <t>ラガシュ クリーミー豆</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>燃料</t>
+          <t>食品</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>apollostation 北海道エネルギー 小樽市内店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D66" s="5" t="n">
-        <v>161.0199714693295</v>
+        <v>798</v>
       </c>
       <c r="E66" s="8" t="n">
         <v>46135</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>R20260423-APOLLO-1702</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>28.04L x 単価166円</t>
+          <t>IMG_8766で追加。商品名は読める範囲</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ロールケーキ(チョコ)</t>
+          <t>リスカ うまい輪チーズ</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -12454,58 +12597,58 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D67" s="5" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>46147</v>
+        <v>46135</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>人参</t>
+          <t>レギュラーガソリン</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>燃料</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>apollostation 北海道エネルギー 小樽市内店</t>
         </is>
       </c>
       <c r="D68" s="5" t="n">
-        <v>188</v>
-      </c>
-      <c r="E68" t="n">
-        <v>46154</v>
+        <v>160.9843081312411</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260423-APOLLO-1702</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>30%値引</t>
+          <t>28.04L x 単価166円（明細照合用に実額4,654円で計上）</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>今川焼(あまおう苺)</t>
+          <t>ロールケーキ(チョコ)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -12519,59 +12662,59 @@
         </is>
       </c>
       <c r="D69" s="5" t="n">
-        <v>164</v>
-      </c>
-      <c r="E69" t="n">
-        <v>46154</v>
+        <v>80</v>
+      </c>
+      <c r="E69" s="8" t="n">
+        <v>46147</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>全粒粉ミニロール</t>
+          <t>人参</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D70" s="5" t="n">
-        <v>278</v>
+        <v>188</v>
       </c>
       <c r="E70" s="8" t="n">
-        <v>46147</v>
+        <v>46154</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260512-COOP</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>30%値引</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>北海道サツラク牛乳</t>
+          <t>今川焼(あまおう苺)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>乳製品</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -12580,153 +12723,148 @@
         </is>
       </c>
       <c r="D71" s="5" t="n">
-        <v>238</v>
-      </c>
-      <c r="E71" t="n">
-        <v>46151</v>
+        <v>164</v>
+      </c>
+      <c r="E71" s="8" t="n">
+        <v>46154</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260512-AEON</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>厚揚げがんばれ!野菜</t>
+          <t>全粒粉ミニロール</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>惣菜・豆腐</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D72" s="5" t="n">
-        <v>138</v>
-      </c>
-      <c r="E72" t="n">
-        <v>46154</v>
+        <v>278</v>
+      </c>
+      <c r="E72" s="8" t="n">
+        <v>46147</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>20%値引</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>厚焼金パンひとり</t>
+          <t>北海道サツラク牛乳</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>乳製品</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ルタオ みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D73" s="5" t="n">
-        <v>388</v>
-      </c>
-      <c r="E73" t="n">
-        <v>46154</v>
+        <v>238</v>
+      </c>
+      <c r="E73" s="8" t="n">
+        <v>46151</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>R20260512-LETAO</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>商品名は画像から読める範囲</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>和風ハンバーグ&amp;あさり</t>
+          <t>厚揚げがんばれ!野菜</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>惣菜・豆腐</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D74" s="5" t="n">
-        <v>299</v>
+        <v>138</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>46152</v>
+        <v>46154</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
+          <t>R20260512-COOP</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>20%値引</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>塩おむすび2個</t>
+          <t>厚焼金パンひとり</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>ルタオ みどり店</t>
         </is>
       </c>
       <c r="D75" s="5" t="n">
-        <v>94</v>
+        <v>388</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>46135</v>
+        <v>46154</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260512-LETAO</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>塩おむすび3個</t>
+          <t>和風ハンバーグ&amp;あさり</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -12740,14 +12878,14 @@
         </is>
       </c>
       <c r="D76" s="5" t="n">
-        <v>139</v>
+        <v>299</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>46135</v>
+        <v>46152</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260510-AEON-1911</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -12759,152 +12897,162 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>塩味ソフト</t>
+          <t>塩おむすび2個</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>イオン マックスバリュ手宮店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D77" s="5" t="n">
-        <v>128</v>
+        <v>94</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>46141</v>
+        <v>46135</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>R20260429-AEON-MAXVALU-1437</t>
+          <t>R20260423-AEON-1917</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>大根</t>
+          <t>塩おむすび3個</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D78" s="5" t="n">
-        <v>198</v>
+        <v>139</v>
       </c>
       <c r="E78" s="8" t="n">
         <v>46135</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260423-AEON-1917</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>大豆のうまみ絹とうふ</t>
+          <t>塩味ソフト</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>豆腐</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>イオン マックスバリュ手宮店</t>
         </is>
       </c>
       <c r="D79" s="5" t="n">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>46135</v>
+        <v>46141</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260429-AEON-MAXVALU-1437</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>山崎スイートバターB5</t>
+          <t>大根</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D80" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="E80" t="n">
-        <v>46151</v>
+        <v>198</v>
+      </c>
+      <c r="E80" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>強炭酸水レモン</t>
+          <t>大豆のうまみ絹とうふ</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>飲料</t>
+          <t>豆腐</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D81" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="E81" t="n">
-        <v>46152</v>
+        <v>98</v>
+      </c>
+      <c r="E81" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>R20260510-GYOMU</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>愛別産イエスななつぼし</t>
+          <t>山崎スイートバターB5</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>米</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -12913,97 +13061,87 @@
         </is>
       </c>
       <c r="D82" s="5" t="n">
-        <v>3584</v>
-      </c>
-      <c r="E82" t="n">
+        <v>100</v>
+      </c>
+      <c r="E82" s="8" t="n">
         <v>46151</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
           <t>R20260509-AEON</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>5kg等の容量は画像から未確認</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>手抜き司盛合せ12貫</t>
+          <t>強炭酸水レモン</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>飲料</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D83" s="5" t="n">
-        <v>349</v>
+        <v>38</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>46146</v>
+        <v>46152</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260510-GYOMU</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>明治ブルガリアヨーグルト</t>
+          <t>愛別産イエスななつぼし</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>乳製品</t>
+          <t>米</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D84" s="5" t="n">
-        <v>158</v>
-      </c>
-      <c r="E84" t="n">
-        <v>46154</v>
+        <v>3584</v>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>46151</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2個 x 単158円</t>
+          <t>5kg等の容量は画像から未確認</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>東ハトふんわり4連</t>
+          <t>手抜き司盛合せ12貫</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>寿司</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -13012,59 +13150,64 @@
         </is>
       </c>
       <c r="D85" s="5" t="n">
-        <v>148</v>
-      </c>
-      <c r="E85" t="n">
-        <v>46151</v>
+        <v>349</v>
+      </c>
+      <c r="E85" s="8" t="n">
+        <v>46146</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>商品名は画像から読める範囲</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>松屋 生沖縄黒飴</t>
+          <t>明治ブルガリアヨーグルト</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>乳製品</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D86" s="5" t="n">
-        <v>185</v>
-      </c>
-      <c r="E86" t="n">
+        <v>158</v>
+      </c>
+      <c r="E86" s="8" t="n">
         <v>46154</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>R20260512-AEON</t>
+          <t>R20260512-COOP</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2個 x 単158円</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>松竹梅卵生貯蔵酒</t>
+          <t>東ハトふんわり4連</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>酒</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -13073,31 +13216,31 @@
         </is>
       </c>
       <c r="D87" s="5" t="n">
-        <v>1350</v>
+        <v>148</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>46139</v>
+        <v>46151</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>10%対象</t>
+          <t>商品名は画像から読める範囲</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>海苔弁当(白身フライ)</t>
+          <t>松屋 生沖縄黒飴</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>弁当</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -13106,31 +13249,26 @@
         </is>
       </c>
       <c r="D88" s="5" t="n">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="E88" s="8" t="n">
-        <v>46139</v>
+        <v>46154</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260512-AEON</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>減塩ひとくち辛子明太子</t>
+          <t>松竹梅卵生貯蔵酒</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>酒</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -13139,7 +13277,7 @@
         </is>
       </c>
       <c r="D89" s="5" t="n">
-        <v>199</v>
+        <v>1350</v>
       </c>
       <c r="E89" s="8" t="n">
         <v>46139</v>
@@ -13151,52 +13289,52 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>10%対象</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>灯油</t>
+          <t>海苔弁当(白身フライ)</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>燃料</t>
+          <t>弁当</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>apollostation 北海道エネルギー 小樽市内店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D90" s="5" t="n">
-        <v>144</v>
-      </c>
-      <c r="E90" t="n">
-        <v>46124</v>
+        <v>199</v>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>46139</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>R20260412-APOLLO</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>41.96L x 単価144円</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>炙りしめサバ握り寿司</t>
+          <t>減塩ひとくち辛子明太子</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -13205,14 +13343,14 @@
         </is>
       </c>
       <c r="D91" s="5" t="n">
-        <v>149</v>
+        <v>199</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>46146</v>
+        <v>46139</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -13224,45 +13362,45 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>焼き菓子</t>
+          <t>灯油</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>燃料</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>apollostation 北海道エネルギー 小樽市内店</t>
         </is>
       </c>
       <c r="D92" s="5" t="n">
-        <v>204</v>
+        <v>144</v>
       </c>
       <c r="E92" s="8" t="n">
-        <v>46135</v>
+        <v>46124</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260412-APOLLO</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>40%値引</t>
+          <t>41.96L x 単価144円</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>焼姫手羽もと(照焼)</t>
+          <t>炙りしめサバ握り寿司</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>寿司</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -13271,14 +13409,14 @@
         </is>
       </c>
       <c r="D93" s="5" t="n">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -13290,12 +13428,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>焼物</t>
+          <t>焼き菓子</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -13304,26 +13442,26 @@
         </is>
       </c>
       <c r="D94" s="5" t="n">
-        <v>187</v>
+        <v>204</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>46147</v>
+        <v>46135</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>40%値引</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>牛カルビさける3種チーズ</t>
+          <t>焼姫手羽もと(照焼)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -13337,14 +13475,14 @@
         </is>
       </c>
       <c r="D95" s="5" t="n">
-        <v>349</v>
+        <v>118</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>46152</v>
+        <v>46139</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -13356,12 +13494,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>牛焼肉</t>
+          <t>焼物</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>肉</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -13370,14 +13508,14 @@
         </is>
       </c>
       <c r="D96" s="5" t="n">
-        <v>292</v>
+        <v>187</v>
       </c>
       <c r="E96" s="8" t="n">
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -13389,12 +13527,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>生くろわっさん</t>
+          <t>牛カルビさける3種チーズ</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -13403,26 +13541,31 @@
         </is>
       </c>
       <c r="D97" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="E97" t="n">
-        <v>46151</v>
+        <v>349</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>46152</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260510-AEON-1911</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>生ます</t>
+          <t>牛焼肉</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>肉</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -13431,14 +13574,14 @@
         </is>
       </c>
       <c r="D98" s="5" t="n">
-        <v>241</v>
-      </c>
-      <c r="E98" t="n">
-        <v>46151</v>
+        <v>292</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>46139</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -13450,12 +13593,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>生乳プレーンヨーグルト</t>
+          <t>生くろわっさん</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>乳製品</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -13464,31 +13607,26 @@
         </is>
       </c>
       <c r="D99" s="5" t="n">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>46135</v>
+        <v>46151</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>20%値引</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>白・桜 うぐいす餅セット</t>
+          <t>生ます</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>和菓子</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -13497,14 +13635,14 @@
         </is>
       </c>
       <c r="D100" s="5" t="n">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="E100" s="8" t="n">
-        <v>46146</v>
+        <v>46151</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -13516,12 +13654,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>真たら</t>
+          <t>生乳プレーンヨーグルト</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>乳製品</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -13530,219 +13668,219 @@
         </is>
       </c>
       <c r="D101" s="5" t="n">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>46139</v>
+        <v>46135</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>20%値引</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>粉末黒糖</t>
+          <t>白・桜 うぐいす餅セット</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>砂糖・甘味料</t>
+          <t>和菓子</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D102" s="5" t="n">
-        <v>548</v>
-      </c>
-      <c r="E102" t="n">
-        <v>46152</v>
+        <v>249</v>
+      </c>
+      <c r="E102" s="8" t="n">
+        <v>46146</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>R20260510-GYOMU</t>
+          <t>R20260504-AEON-1918</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>若キャラメルローストビ</t>
+          <t>真たら</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D103" s="5" t="n">
-        <v>98</v>
+        <v>138</v>
       </c>
       <c r="E103" s="8" t="n">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>商品名は判読不確実</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>菊田堂さんとうふ</t>
+          <t>粉末黒糖</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>豆腐</t>
+          <t>砂糖・甘味料</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D104" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="E104" t="n">
-        <v>46154</v>
+        <v>548</v>
+      </c>
+      <c r="E104" s="8" t="n">
+        <v>46152</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>150円に訂正</t>
+          <t>R20260510-GYOMU</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>評判屋 せき止め飴</t>
+          <t>若キャラメルローストビ</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>医薬・日用品</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>サンドラッグ 小樽稲穂店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D105" s="5" t="n">
-        <v>300</v>
+        <v>98</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>46152</v>
+        <v>46135</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>R20260510-SUNDRUG-1326</t>
+          <t>R20260423-GYOMU-1651</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>豚しゃぶしゃぶ用</t>
+          <t>菊田堂さんとうふ</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>肉</t>
+          <t>豆腐</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D106" s="5" t="n">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="E106" s="8" t="n">
-        <v>46147</v>
+        <v>46154</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260512-COOP</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>150円に訂正</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>豚肉とんかつ用</t>
+          <t>評判屋 せき止め飴</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>肉</t>
+          <t>医薬・日用品</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>サンドラッグ 小樽稲穂店</t>
         </is>
       </c>
       <c r="D107" s="5" t="n">
-        <v>327</v>
+        <v>300</v>
       </c>
       <c r="E107" s="8" t="n">
         <v>46152</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260510-SUNDRUG-1326</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>超熟フォカッチャ3個入</t>
+          <t>豚しゃぶしゃぶ用</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>肉</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -13751,26 +13889,31 @@
         </is>
       </c>
       <c r="D108" s="5" t="n">
-        <v>200</v>
+        <v>159</v>
       </c>
       <c r="E108" s="8" t="n">
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260505-AEON-1930</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>超熟北海道食パン</t>
+          <t>豚肉とんかつ用</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>肉</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -13779,54 +13922,59 @@
         </is>
       </c>
       <c r="D109" s="5" t="n">
-        <v>240</v>
+        <v>327</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>46135</v>
+        <v>46152</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260510-AEON-1911</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>長芋</t>
+          <t>超熟フォカッチャ3個入</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D110" s="5" t="n">
-        <v>278</v>
+        <v>200</v>
       </c>
       <c r="E110" s="8" t="n">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>隔らる！大きな肉焼売</t>
+          <t>超熟北海道食パン</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -13835,87 +13983,87 @@
         </is>
       </c>
       <c r="D111" s="5" t="n">
-        <v>149</v>
+        <v>240</v>
       </c>
       <c r="E111" s="8" t="n">
-        <v>46146</v>
+        <v>46135</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>50%値引。商品名は判読不確実</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>雪印 北海道バター</t>
+          <t>長芋</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>乳製品</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D112" s="5" t="n">
-        <v>398</v>
-      </c>
-      <c r="E112" t="n">
-        <v>46151</v>
+        <v>278</v>
+      </c>
+      <c r="E112" s="8" t="n">
+        <v>46135</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>韓国ハッピーターン</t>
+          <t>隔らる！大きな肉焼売</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D113" s="5" t="n">
-        <v>88</v>
+        <v>149</v>
       </c>
       <c r="E113" s="8" t="n">
-        <v>46135</v>
+        <v>46146</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260504-AEON-1918</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>50%値引。商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>魚屋の寿司</t>
+          <t>雪印 北海道バター</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>乳製品</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -13924,50 +14072,106 @@
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>499</v>
+        <v>398</v>
       </c>
       <c r="E114" s="8" t="n">
-        <v>46139</v>
+        <v>46151</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>魚屋の海鮮ちらし</t>
+          <t>韓国ハッピーターン</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D115" s="5" t="n">
-        <v>249</v>
+        <v>88</v>
       </c>
       <c r="E115" s="8" t="n">
         <v>46135</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
+          <t>R20260423-GYOMU-1651</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>魚屋の寿司</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>寿司</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>イオン小樽店</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="n">
+        <v>499</v>
+      </c>
+      <c r="E116" s="8" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>50%値引</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>魚屋の海鮮ちらし</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>寿司</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>イオン小樽店</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="n">
+        <v>249</v>
+      </c>
+      <c r="E117" s="8" t="n">
+        <v>46135</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
           <t>R20260423-AEON-1917</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr">
+      <c r="G117" t="inlineStr">
         <is>
           <t>50%値引</t>
         </is>

</xml_diff>

<commit_message>
Correct CanDo receipt amount display
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -3502,19 +3502,19 @@
         <v>2</v>
       </c>
       <c r="I48" s="5" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="J48" s="5" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="K48" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L48" s="5" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="M48" s="5" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="N48" t="n">
         <v>0.1</v>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2個</t>
+          <t>2個、税込合計220円に訂正</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -9847,7 +9847,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="F9" t="n">
         <v>0.1</v>
@@ -9870,7 +9870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>B5ノート 2個。</t>
+          <t>B5ノート 2個。税込220円に訂正。</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -10503,7 +10503,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>47057</v>
+        <v>47077</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
@@ -10619,7 +10619,7 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>46135</v>
@@ -10631,7 +10631,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2個</t>
+          <t>2個、税込合計220円に訂正</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Gyomu May 10 total
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -288,7 +288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q135"/>
+  <dimension ref="A1:Q136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -9370,6 +9370,75 @@
       <c r="Q135" t="inlineStr">
         <is>
           <t>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>R20260510-GYOMU</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="n">
+        <v>46152</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>業務スーパー 小樽店</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>消費税等</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>税</t>
+        </is>
+      </c>
+      <c r="H136" t="n">
+        <v>1</v>
+      </c>
+      <c r="I136" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="J136" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="K136" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L136" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="M136" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>税込合計1,179円に合わせるため追加</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>receipt_images/R20260510-GYOMU_IMG_8757.JPG</t>
         </is>
       </c>
     </row>
@@ -9587,7 +9656,7 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>1092</v>
+        <v>1179</v>
       </c>
       <c r="F4" t="n">
         <v>0.08</v>
@@ -9610,7 +9679,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>CARDNET控えは同じ購入のカード控えとして扱い、二重計上しない。</t>
+          <t>税込支払額1,179円に訂正。消費税等87円を明細に追加。</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -10477,7 +10546,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -10503,7 +10572,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>47077</v>
+        <v>47164</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
@@ -10520,7 +10589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -13329,111 +13398,111 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>減塩ひとくち辛子明太子</t>
+          <t>消費税等</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>税</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D91" s="5" t="n">
-        <v>199</v>
+        <v>87</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>46139</v>
+        <v>46152</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260510-GYOMU</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>税込合計1,179円に合わせるため追加</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>灯油</t>
+          <t>減塩ひとくち辛子明太子</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>燃料</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>apollostation 北海道エネルギー 小樽市内店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D92" s="5" t="n">
-        <v>144</v>
+        <v>199</v>
       </c>
       <c r="E92" s="8" t="n">
-        <v>46124</v>
+        <v>46139</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>R20260412-APOLLO</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>41.96L x 単価144円</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>炙りしめサバ握り寿司</t>
+          <t>灯油</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>燃料</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>apollostation 北海道エネルギー 小樽市内店</t>
         </is>
       </c>
       <c r="D93" s="5" t="n">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>46146</v>
+        <v>46124</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260412-APOLLO</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>41.96L x 単価144円</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>焼き菓子</t>
+          <t>炙りしめサバ握り寿司</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>寿司</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -13442,31 +13511,31 @@
         </is>
       </c>
       <c r="D94" s="5" t="n">
-        <v>204</v>
+        <v>149</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>46135</v>
+        <v>46146</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>40%値引</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>焼姫手羽もと(照焼)</t>
+          <t>焼き菓子</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -13475,26 +13544,26 @@
         </is>
       </c>
       <c r="D95" s="5" t="n">
-        <v>118</v>
+        <v>204</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>46139</v>
+        <v>46135</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>40%値引</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>焼物</t>
+          <t>焼姫手羽もと(照焼)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -13508,14 +13577,14 @@
         </is>
       </c>
       <c r="D96" s="5" t="n">
-        <v>187</v>
+        <v>118</v>
       </c>
       <c r="E96" s="8" t="n">
-        <v>46147</v>
+        <v>46139</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -13527,7 +13596,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>牛カルビさける3種チーズ</t>
+          <t>焼物</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -13541,14 +13610,14 @@
         </is>
       </c>
       <c r="D97" s="5" t="n">
-        <v>349</v>
+        <v>187</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>46152</v>
+        <v>46147</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -13560,12 +13629,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>牛焼肉</t>
+          <t>牛カルビさける3種チーズ</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>肉</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -13574,14 +13643,14 @@
         </is>
       </c>
       <c r="D98" s="5" t="n">
-        <v>292</v>
+        <v>349</v>
       </c>
       <c r="E98" s="8" t="n">
-        <v>46139</v>
+        <v>46152</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260510-AEON-1911</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -13593,12 +13662,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>生くろわっさん</t>
+          <t>牛焼肉</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>肉</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -13607,26 +13676,31 @@
         </is>
       </c>
       <c r="D99" s="5" t="n">
-        <v>120</v>
+        <v>292</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>46151</v>
+        <v>46139</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>生ます</t>
+          <t>生くろわっさん</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -13635,7 +13709,7 @@
         </is>
       </c>
       <c r="D100" s="5" t="n">
-        <v>241</v>
+        <v>120</v>
       </c>
       <c r="E100" s="8" t="n">
         <v>46151</v>
@@ -13645,21 +13719,16 @@
           <t>R20260509-AEON</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>50%値引</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>生乳プレーンヨーグルト</t>
+          <t>生ます</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>乳製品</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -13668,31 +13737,31 @@
         </is>
       </c>
       <c r="D101" s="5" t="n">
-        <v>158</v>
+        <v>241</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>46135</v>
+        <v>46151</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>20%値引</t>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>白・桜 うぐいす餅セット</t>
+          <t>生乳プレーンヨーグルト</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>和菓子</t>
+          <t>乳製品</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -13701,31 +13770,31 @@
         </is>
       </c>
       <c r="D102" s="5" t="n">
-        <v>249</v>
+        <v>158</v>
       </c>
       <c r="E102" s="8" t="n">
-        <v>46146</v>
+        <v>46135</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>50%値引</t>
+          <t>20%値引</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>真たら</t>
+          <t>白・桜 うぐいす餅セット</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>魚介</t>
+          <t>和菓子</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -13734,14 +13803,14 @@
         </is>
       </c>
       <c r="D103" s="5" t="n">
-        <v>138</v>
+        <v>249</v>
       </c>
       <c r="E103" s="8" t="n">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260504-AEON-1918</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -13753,40 +13822,45 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>粉末黒糖</t>
+          <t>真たら</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>砂糖・甘味料</t>
+          <t>魚介</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D104" s="5" t="n">
-        <v>548</v>
+        <v>138</v>
       </c>
       <c r="E104" s="8" t="n">
-        <v>46152</v>
+        <v>46139</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>R20260510-GYOMU</t>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>若キャラメルローストビ</t>
+          <t>粉末黒糖</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>砂糖・甘味料</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -13795,120 +13869,115 @@
         </is>
       </c>
       <c r="D105" s="5" t="n">
-        <v>98</v>
+        <v>548</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>46135</v>
+        <v>46152</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>商品名は判読不確実</t>
+          <t>R20260510-GYOMU</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>菊田堂さんとうふ</t>
+          <t>若キャラメルローストビ</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>豆腐</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>COOP SAPPORO みどり店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D106" s="5" t="n">
-        <v>150</v>
+        <v>98</v>
       </c>
       <c r="E106" s="8" t="n">
-        <v>46154</v>
+        <v>46135</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>R20260512-COOP</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>150円に訂正</t>
+          <t>商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>評判屋 せき止め飴</t>
+          <t>菊田堂さんとうふ</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>医薬・日用品</t>
+          <t>豆腐</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>サンドラッグ 小樽稲穂店</t>
+          <t>COOP SAPPORO みどり店</t>
         </is>
       </c>
       <c r="D107" s="5" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>46152</v>
+        <v>46154</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>R20260510-SUNDRUG-1326</t>
+          <t>R20260512-COOP</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>150円に訂正</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>豚しゃぶしゃぶ用</t>
+          <t>評判屋 せき止め飴</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>肉</t>
+          <t>医薬・日用品</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>サンドラッグ 小樽稲穂店</t>
         </is>
       </c>
       <c r="D108" s="5" t="n">
-        <v>159</v>
+        <v>300</v>
       </c>
       <c r="E108" s="8" t="n">
-        <v>46147</v>
+        <v>46152</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>R20260505-AEON-1930</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260510-SUNDRUG-1326</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>豚肉とんかつ用</t>
+          <t>豚しゃぶしゃぶ用</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -13922,14 +13991,14 @@
         </is>
       </c>
       <c r="D109" s="5" t="n">
-        <v>327</v>
+        <v>159</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>46152</v>
+        <v>46147</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>R20260510-AEON-1911</t>
+          <t>R20260505-AEON-1930</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -13941,12 +14010,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>超熟フォカッチャ3個入</t>
+          <t>豚肉とんかつ用</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>肉</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -13955,21 +14024,26 @@
         </is>
       </c>
       <c r="D110" s="5" t="n">
-        <v>200</v>
+        <v>327</v>
       </c>
       <c r="E110" s="8" t="n">
-        <v>46139</v>
+        <v>46152</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
+          <t>R20260510-AEON-1911</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>50%値引</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>超熟北海道食パン</t>
+          <t>超熟フォカッチャ3個入</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -13983,87 +14057,82 @@
         </is>
       </c>
       <c r="D111" s="5" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="E111" s="8" t="n">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>R20260423-AEON-1917</t>
+          <t>R20260427-AEON-1920</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>長芋</t>
+          <t>超熟北海道食パン</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D112" s="5" t="n">
-        <v>278</v>
+        <v>240</v>
       </c>
       <c r="E112" s="8" t="n">
         <v>46135</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260423-AEON-1917</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>隔らる！大きな肉焼売</t>
+          <t>長芋</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>惣菜</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D113" s="5" t="n">
-        <v>149</v>
+        <v>278</v>
       </c>
       <c r="E113" s="8" t="n">
-        <v>46146</v>
+        <v>46135</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>R20260504-AEON-1918</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>50%値引。商品名は判読不確実</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>雪印 北海道バター</t>
+          <t>隔らる！大きな肉焼売</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>乳製品</t>
+          <t>惣菜</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -14072,106 +14141,139 @@
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>398</v>
+        <v>149</v>
       </c>
       <c r="E114" s="8" t="n">
-        <v>46151</v>
+        <v>46146</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>R20260509-AEON</t>
+          <t>R20260504-AEON-1918</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>50%値引。商品名は判読不確実</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>韓国ハッピーターン</t>
+          <t>雪印 北海道バター</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>菓子</t>
+          <t>乳製品</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>業務スーパー 小樽店</t>
+          <t>イオン小樽店</t>
         </is>
       </c>
       <c r="D115" s="5" t="n">
-        <v>88</v>
+        <v>398</v>
       </c>
       <c r="E115" s="8" t="n">
-        <v>46135</v>
+        <v>46151</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>R20260423-GYOMU-1651</t>
+          <t>R20260509-AEON</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>魚屋の寿司</t>
+          <t>韓国ハッピーターン</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>寿司</t>
+          <t>菓子</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>イオン小樽店</t>
+          <t>業務スーパー 小樽店</t>
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>499</v>
+        <v>88</v>
       </c>
       <c r="E116" s="8" t="n">
-        <v>46139</v>
+        <v>46135</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>R20260427-AEON-1920</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>50%値引</t>
+          <t>R20260423-GYOMU-1651</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>魚屋の寿司</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>寿司</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>イオン小樽店</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="n">
+        <v>499</v>
+      </c>
+      <c r="E117" s="8" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>R20260427-AEON-1920</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>50%値引</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>魚屋の海鮮ちらし</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>寿司</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>イオン小樽店</t>
-        </is>
-      </c>
-      <c r="D117" s="5" t="n">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>イオン小樽店</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="n">
         <v>249</v>
       </c>
-      <c r="E117" s="8" t="n">
+      <c r="E118" s="8" t="n">
         <v>46135</v>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F118" t="inlineStr">
         <is>
           <t>R20260423-AEON-1917</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="G118" t="inlineStr">
         <is>
           <t>50%値引</t>
         </is>

</xml_diff>

<commit_message>
Show only tax-included totals
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R7aeccbb56e7745e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R94de0b9cf1044342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="Reaa77990ccc74b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R567f4f6f45844984"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R7ffca4e2553e4d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R3ad1d18ae6c8478b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9537,7 +9537,7 @@
         </x:is>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>税込金額</x:v>
+        <x:v>税込合計</x:v>
       </x:c>
       <x:c r="F1" s="3" t="inlineStr">
         <x:is>
@@ -10572,7 +10572,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>税込金額合計</x:v>
+        <x:v>税込合計</x:v>
       </x:c>
       <x:c r="B25" s="7" t="n">
         <x:v>49528</x:v>

</xml_diff>

<commit_message>
Keep only tax-included total display
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R567f4f6f45844984"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R7ffca4e2553e4d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R3ad1d18ae6c8478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R63c0fddc2da44fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="Rdfd8518cab3e4e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R3591e3cb47564539"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9516,1070 +9516,707 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">レシートID</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">購入日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">時刻</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">店舗</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="A1" t="str">
+        <x:v>レシートID</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>購入日</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>時刻</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>店舗</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
         <x:v>税込合計</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">税率</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">消費税</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">支払合計(税込)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">支払方法</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">読取信頼度</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">備考</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L1" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">画像</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>支払方法</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>読取信頼度</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>備考</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>画像</x:v>
+      </x:c>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
+      <x:c r="L1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260509-AEON</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="7" t="n">
+      <x:c r="A2" t="str">
+        <x:v>R20260509-AEON</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
         <x:v>46151</x:v>
       </x:c>
-      <x:c r="C2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:22</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E2" s="5" t="n">
+      <x:c r="C2" t="str">
+        <x:v>19:22</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E2" t="n">
         <x:v>6923</x:v>
       </x:c>
-      <x:c r="F2" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="n">
-        <x:v>512</x:v>
-      </x:c>
-      <x:c r="H2" s="5" t="n">
-        <x:v>6923</x:v>
-      </x:c>
-      <x:c r="I2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K2" t="str">
+      <x:c r="F2" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
         <x:v>税込合計6,923円に統一。消費税等512円を明細に追加。</x:v>
       </x:c>
-      <x:c r="L2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260509-AEON_IMG_8759.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>receipt_images/R20260509-AEON_IMG_8759.JPG</x:v>
+      </x:c>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260512-AEON</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="7" t="n">
+      <x:c r="A3" t="str">
+        <x:v>R20260512-AEON</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
         <x:v>46154</x:v>
       </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:17</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="5" t="n">
+      <x:c r="C3" t="str">
+        <x:v>19:17</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E3" t="n">
         <x:v>1355</x:v>
       </x:c>
-      <x:c r="F3" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G3" s="5" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="H3" s="5" t="n">
-        <x:v>1355</x:v>
-      </x:c>
-      <x:c r="I3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K3" t="str">
+      <x:c r="F3" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
         <x:v>今川焼は50%値引後で実質単価を算出。</x:v>
       </x:c>
-      <x:c r="L3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260512-AEON_IMG_8757.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>receipt_images/R20260512-AEON_IMG_8757.JPG</x:v>
+      </x:c>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260510-GYOMU</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="7" t="n">
+      <x:c r="A4" t="str">
+        <x:v>R20260510-GYOMU</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
         <x:v>46152</x:v>
       </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">13:25</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">業務スーパー 小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="5" t="n">
+      <x:c r="C4" t="str">
+        <x:v>13:25</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>業務スーパー 小樽店</x:v>
+      </x:c>
+      <x:c r="E4" t="n">
         <x:v>1179</x:v>
       </x:c>
-      <x:c r="F4" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="n">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="H4" s="5" t="n">
-        <x:v>1179</x:v>
-      </x:c>
-      <x:c r="I4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K4" t="str">
+      <x:c r="F4" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
         <x:v>税込支払額1,179円に訂正。消費税等87円を明細に追加。</x:v>
       </x:c>
-      <x:c r="L4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260510-GYOMU_IMG_8757.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>receipt_images/R20260510-GYOMU_IMG_8757.JPG</x:v>
+      </x:c>
+      <x:c r="J4"/>
+      <x:c r="K4"/>
+      <x:c r="L4"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260512-LETAO</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="7" t="n">
+      <x:c r="A5" t="str">
+        <x:v>R20260512-LETAO</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
         <x:v>46154</x:v>
       </x:c>
-      <x:c r="C5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15:51</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ルタオ みどり店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="5" t="n">
+      <x:c r="C5" t="str">
+        <x:v>15:51</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>ルタオ みどり店</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
         <x:v>388</x:v>
       </x:c>
-      <x:c r="F5" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G5" s="5" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="H5" s="5" t="n">
-        <x:v>388</x:v>
-      </x:c>
-      <x:c r="I5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">JCB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K5" t="str">
+      <x:c r="F5" t="str">
+        <x:v>JCB</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
         <x:v>商品名はレシート画像から読める範囲。内消費税28円。</x:v>
       </x:c>
-      <x:c r="L5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260512-LETAO_IMG_8760.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>receipt_images/R20260512-LETAO_IMG_8760.JPG</x:v>
+      </x:c>
+      <x:c r="J5"/>
+      <x:c r="K5"/>
+      <x:c r="L5"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260512-COOP</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="7" t="n">
+      <x:c r="A6" t="str">
+        <x:v>R20260512-COOP</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
         <x:v>46154</x:v>
       </x:c>
-      <x:c r="C6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:04</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">COOP SAPPORO みどり店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="5" t="n">
+      <x:c r="C6" t="str">
+        <x:v>16:04</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>COOP SAPPORO みどり店</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
         <x:v>2201</x:v>
       </x:c>
-      <x:c r="F6" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="n">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="H6" s="5" t="n">
-        <x:v>2201</x:v>
-      </x:c>
-      <x:c r="I6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K6" t="str">
+      <x:c r="F6" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
         <x:v>領収書。値引は読取可能範囲で反映。税込合計2,201円。</x:v>
       </x:c>
-      <x:c r="L6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260512-COOP_IMG_8760.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>receipt_images/R20260512-COOP_IMG_8760.JPG</x:v>
+      </x:c>
+      <x:c r="J6"/>
+      <x:c r="K6"/>
+      <x:c r="L6"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260412-APOLLO</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="7" t="n">
+      <x:c r="A7" t="str">
+        <x:v>R20260412-APOLLO</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
         <x:v>46124</x:v>
       </x:c>
-      <x:c r="C7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">13:05</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">apollostation 北海道エネルギー 小樽市内店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" s="5" t="n">
+      <x:c r="C7" t="str">
+        <x:v>13:05</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>apollostation 北海道エネルギー 小樽市内店</x:v>
+      </x:c>
+      <x:c r="E7" t="n">
         <x:v>6042</x:v>
       </x:c>
-      <x:c r="F7" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="G7" s="5" t="n">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="n">
-        <x:v>6042</x:v>
-      </x:c>
-      <x:c r="I7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K7" t="str">
+      <x:c r="F7" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
         <x:v>灯油 41.96L、単価144円。内税10%対象。</x:v>
       </x:c>
-      <x:c r="L7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260412-APOLLO_IMG_8761_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>receipt_images/R20260412-APOLLO_IMG_8761_2.JPG</x:v>
+      </x:c>
+      <x:c r="J7"/>
+      <x:c r="K7"/>
+      <x:c r="L7"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260423-AEON-1917</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="7" t="n">
+      <x:c r="A8" t="str">
+        <x:v>R20260423-AEON-1917</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
         <x:v>46135</x:v>
       </x:c>
-      <x:c r="C8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:17</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" s="5" t="n">
+      <x:c r="C8" t="str">
+        <x:v>19:17</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
         <x:v>2124</x:v>
       </x:c>
-      <x:c r="F8" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="n">
-        <x:v>157</x:v>
-      </x:c>
-      <x:c r="H8" s="5" t="n">
-        <x:v>2124</x:v>
-      </x:c>
-      <x:c r="I8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K8" t="str">
+      <x:c r="F8" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
         <x:v>IMG_8765左。明細合計一致。</x:v>
       </x:c>
-      <x:c r="L8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260423-AEON-1917_IMG_8765.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>receipt_images/R20260423-AEON-1917_IMG_8765.JPG</x:v>
+      </x:c>
+      <x:c r="J8"/>
+      <x:c r="K8"/>
+      <x:c r="L8"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260423-CANDO-1602</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="7" t="n">
+      <x:c r="A9" t="str">
+        <x:v>R20260423-CANDO-1602</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
         <x:v>46135</x:v>
       </x:c>
-      <x:c r="C9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CanDo DCM手宮店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="5" t="n">
+      <x:c r="C9" t="str">
+        <x:v>16:02</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>CanDo DCM手宮店</x:v>
+      </x:c>
+      <x:c r="E9" t="n">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="F9" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="G9" s="5" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H9" s="5" t="n">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="I9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">現金</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K9" t="str">
+      <x:c r="F9" t="str">
+        <x:v>現金</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
         <x:v>B5ノート 2個。税込220円に訂正。</x:v>
       </x:c>
-      <x:c r="L9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260423-CANDO-1602_IMG_8765.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>receipt_images/R20260423-CANDO-1602_IMG_8765.JPG</x:v>
+      </x:c>
+      <x:c r="J9"/>
+      <x:c r="K9"/>
+      <x:c r="L9"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260510-SUNDRUG-1326</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="7" t="n">
+      <x:c r="A10" t="str">
+        <x:v>R20260510-SUNDRUG-1326</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
         <x:v>46152</x:v>
       </x:c>
-      <x:c r="C10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">13:26</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">サンドラッグ 小樽稲穂店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="5" t="n">
+      <x:c r="C10" t="str">
+        <x:v>13:26</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>サンドラッグ 小樽稲穂店</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
         <x:v>535</x:v>
       </x:c>
-      <x:c r="F10" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H10" s="5" t="n">
-        <x:v>535</x:v>
-      </x:c>
-      <x:c r="I10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K10" t="str">
+      <x:c r="F10" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
         <x:v>税込合計535円。</x:v>
       </x:c>
-      <x:c r="L10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260510-SUNDRUG-1326_IMG_8765.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>receipt_images/R20260510-SUNDRUG-1326_IMG_8765.JPG</x:v>
+      </x:c>
+      <x:c r="J10"/>
+      <x:c r="K10"/>
+      <x:c r="L10"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260510-AEON-1911</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="7" t="n">
+      <x:c r="A11" t="str">
+        <x:v>R20260510-AEON-1911</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
         <x:v>46152</x:v>
       </x:c>
-      <x:c r="C11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:11</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E11" s="5" t="n">
+      <x:c r="C11" t="str">
+        <x:v>19:11</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
         <x:v>1578</x:v>
       </x:c>
-      <x:c r="F11" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G11" s="5" t="n">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="H11" s="5" t="n">
-        <x:v>1578</x:v>
-      </x:c>
-      <x:c r="I11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K11" t="str">
+      <x:c r="F11" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
         <x:v>IMG_8765中央右。明細合計一致。</x:v>
       </x:c>
-      <x:c r="L11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260510-AEON-1911_IMG_8765.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>receipt_images/R20260510-AEON-1911_IMG_8765.JPG</x:v>
+      </x:c>
+      <x:c r="J11"/>
+      <x:c r="K11"/>
+      <x:c r="L11"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260505-AEON-1930</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="7" t="n">
+      <x:c r="A12" t="str">
+        <x:v>R20260505-AEON-1930</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
         <x:v>46147</x:v>
       </x:c>
-      <x:c r="C12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:30</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="5" t="n">
+      <x:c r="C12" t="str">
+        <x:v>19:30</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
         <x:v>2744</x:v>
       </x:c>
-      <x:c r="F12" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G12" s="5" t="n">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="H12" s="5" t="n">
-        <x:v>2744</x:v>
-      </x:c>
-      <x:c r="I12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K12" t="str">
+      <x:c r="F12" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
         <x:v>IMG_8765右。明細合計一致。</x:v>
       </x:c>
-      <x:c r="L12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260505-AEON-1930_IMG_8765.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>receipt_images/R20260505-AEON-1930_IMG_8765.JPG</x:v>
+      </x:c>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
+      <x:c r="L12"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260429-AEON-MAXVALU-1437</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="7" t="n">
+      <x:c r="A13" t="str">
+        <x:v>R20260429-AEON-MAXVALU-1437</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
         <x:v>46141</x:v>
       </x:c>
-      <x:c r="C13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14:37</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン マックスバリュ手宮店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E13" s="5" t="n">
+      <x:c r="C13" t="str">
+        <x:v>14:37</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>イオン マックスバリュ手宮店</x:v>
+      </x:c>
+      <x:c r="E13" t="n">
         <x:v>705</x:v>
       </x:c>
-      <x:c r="F13" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G13" s="5" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="H13" s="5" t="n">
-        <x:v>705</x:v>
-      </x:c>
-      <x:c r="I13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">低</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K13" t="str">
+      <x:c r="F13" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>低</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
         <x:v>IMG_8764左。明細読取に差額あり。</x:v>
       </x:c>
-      <x:c r="L13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260429-AEON-MAXVALU-1437_IMG_8764_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>receipt_images/R20260429-AEON-MAXVALU-1437_IMG_8764_2.JPG</x:v>
+      </x:c>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+      <x:c r="L13"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260429-AEON-1746</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" s="7" t="n">
+      <x:c r="A14" t="str">
+        <x:v>R20260429-AEON-1746</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
         <x:v>46141</x:v>
       </x:c>
-      <x:c r="C14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17:46</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E14" s="5" t="n">
+      <x:c r="C14" t="str">
+        <x:v>17:46</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E14" t="n">
         <x:v>555</x:v>
       </x:c>
-      <x:c r="F14" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G14" s="5" t="n">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="H14" s="5" t="n">
-        <x:v>555</x:v>
-      </x:c>
-      <x:c r="I14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K14" t="str">
+      <x:c r="F14" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
         <x:v>明細合計一致。</x:v>
       </x:c>
-      <x:c r="L14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260429-AEON-1746_IMG_8764_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>receipt_images/R20260429-AEON-1746_IMG_8764_2.JPG</x:v>
+      </x:c>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+      <x:c r="L14"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260427-AEON-1920</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="7" t="n">
+      <x:c r="A15" t="str">
+        <x:v>R20260427-AEON-1920</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
         <x:v>46139</x:v>
       </x:c>
-      <x:c r="C15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:20</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E15" s="5" t="n">
+      <x:c r="C15" t="str">
+        <x:v>19:20</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="F15" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G15" s="5" t="n">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="H15" s="5" t="n">
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="I15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K15" t="str">
+      <x:c r="F15" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
         <x:v>8%対象4,181円、10%対象1,350円。明細合計一致。</x:v>
       </x:c>
-      <x:c r="L15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260427-AEON-1920_IMG_8764_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>receipt_images/R20260427-AEON-1920_IMG_8764_2.JPG</x:v>
+      </x:c>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+      <x:c r="L15"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260423-APOLLO-1702</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="7" t="n">
+      <x:c r="A16" t="str">
+        <x:v>R20260423-APOLLO-1702</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
         <x:v>46135</x:v>
       </x:c>
-      <x:c r="C16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17:02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">apollostation 北海道エネルギー 小樽市内店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E16" s="5" t="n">
+      <x:c r="C16" t="str">
+        <x:v>17:02</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>apollostation 北海道エネルギー 小樽市内店</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
         <x:v>4514</x:v>
       </x:c>
-      <x:c r="F16" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="G16" s="5" t="n">
-        <x:v>410</x:v>
-      </x:c>
-      <x:c r="H16" s="5" t="n">
-        <x:v>4514</x:v>
-      </x:c>
-      <x:c r="I16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K16" t="str">
+      <x:c r="F16" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
         <x:v>レギュラーガソリン 28.04L、単価166円、値引140円。</x:v>
       </x:c>
-      <x:c r="L16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260423-APOLLO-1702_IMG_8764_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>receipt_images/R20260423-APOLLO-1702_IMG_8764_2.JPG</x:v>
+      </x:c>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260504-AEON-1918</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="7" t="n">
+      <x:c r="A17" t="str">
+        <x:v>R20260504-AEON-1918</x:v>
+      </x:c>
+      <x:c r="B17" t="n">
         <x:v>46146</x:v>
       </x:c>
-      <x:c r="C17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19:18</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">イオン小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E17" s="5" t="n">
+      <x:c r="C17" t="str">
+        <x:v>19:18</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>イオン小樽店</x:v>
+      </x:c>
+      <x:c r="E17" t="n">
         <x:v>4498</x:v>
       </x:c>
-      <x:c r="F17" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G17" s="5" t="n">
-        <x:v>333</x:v>
-      </x:c>
-      <x:c r="H17" s="5" t="n">
-        <x:v>4498</x:v>
-      </x:c>
-      <x:c r="I17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K17" t="str">
+      <x:c r="F17" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
         <x:v>IMG_8763左。明細合計一致。</x:v>
       </x:c>
-      <x:c r="L17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260504-AEON-1918_IMG_8763_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>receipt_images/R20260504-AEON-1918_IMG_8763_2.JPG</x:v>
+      </x:c>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260423-GYOMU-1651</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="7" t="n">
+      <x:c r="A18" t="str">
+        <x:v>R20260423-GYOMU-1651</x:v>
+      </x:c>
+      <x:c r="B18" t="n">
         <x:v>46135</x:v>
       </x:c>
-      <x:c r="C18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:51</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">業務スーパー 小樽店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E18" s="5" t="n">
+      <x:c r="C18" t="str">
+        <x:v>16:51</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>業務スーパー 小樽店</x:v>
+      </x:c>
+      <x:c r="E18" t="n">
         <x:v>3965</x:v>
       </x:c>
-      <x:c r="F18" t="n">
-        <x:v>0.08</x:v>
-      </x:c>
-      <x:c r="G18" s="5" t="n">
-        <x:v>294</x:v>
-      </x:c>
-      <x:c r="H18" s="5" t="n">
-        <x:v>3965</x:v>
-      </x:c>
-      <x:c r="I18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K18" t="str">
+      <x:c r="F18" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
         <x:v>IMG_8766で再確認。明細合計一致。</x:v>
       </x:c>
-      <x:c r="L18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</x:v>
+      </x:c>
+      <x:c r="J18"/>
+      <x:c r="K18"/>
+      <x:c r="L18"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260429-NISHIMATSUYA-1518</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B19" s="7" t="n">
+      <x:c r="A19" t="str">
+        <x:v>R20260429-NISHIMATSUYA-1518</x:v>
+      </x:c>
+      <x:c r="B19" t="n">
         <x:v>46141</x:v>
       </x:c>
-      <x:c r="C19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15:18</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">西松屋 小樽有幌店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E19" s="5" t="n">
+      <x:c r="C19" t="str">
+        <x:v>15:18</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>西松屋 小樽有幌店</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
         <x:v>966</x:v>
       </x:c>
-      <x:c r="F19" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="G19" s="5" t="n">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="H19" s="5" t="n">
-        <x:v>966</x:v>
-      </x:c>
-      <x:c r="I19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K19" t="str">
+      <x:c r="F19" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
         <x:v>商品名は画像から読める範囲。</x:v>
       </x:c>
-      <x:c r="L19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260429-NISHIMATSUYA-1518_IMG_8763_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>receipt_images/R20260429-NISHIMATSUYA-1518_IMG_8763_2.JPG</x:v>
+      </x:c>
+      <x:c r="J19"/>
+      <x:c r="K19"/>
+      <x:c r="L19"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R20260423-DCM-1619</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B20" s="7" t="n">
+      <x:c r="A20" t="str">
+        <x:v>R20260423-DCM-1619</x:v>
+      </x:c>
+      <x:c r="B20" t="n">
         <x:v>46135</x:v>
       </x:c>
-      <x:c r="C20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:19</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DCM 手宮店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E20" s="5" t="n">
+      <x:c r="C20" t="str">
+        <x:v>16:19</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>DCM 手宮店</x:v>
+      </x:c>
+      <x:c r="E20" t="n">
         <x:v>3036</x:v>
       </x:c>
-      <x:c r="F20" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="G20" s="5" t="n">
-        <x:v>276</x:v>
-      </x:c>
-      <x:c r="H20" s="5" t="n">
-        <x:v>3036</x:v>
-      </x:c>
-      <x:c r="I20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クレジット</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K20" t="str">
+      <x:c r="F20" t="str">
+        <x:v>クレジット</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
         <x:v>税込合計3,036円。</x:v>
       </x:c>
-      <x:c r="L20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">receipt_images/R20260423-DCM-1619_IMG_8763_2.JPG</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>receipt_images/R20260423-DCM-1619_IMG_8763_2.JPG</x:v>
+      </x:c>
+      <x:c r="J20"/>
+      <x:c r="K20"/>
+      <x:c r="L20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="B21" s="7" t="n"/>
-      <x:c r="E21" s="5" t="n"/>
-      <x:c r="G21" s="5" t="n"/>
-      <x:c r="H21" s="5" t="n"/>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">レシート枚数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B22" s="7" t="n">
+      <x:c r="A22" t="str">
+        <x:v>レシート枚数</x:v>
+      </x:c>
+      <x:c r="B22" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="E22" s="5" t="n"/>
-      <x:c r="G22" s="5" t="n"/>
-      <x:c r="H22" s="5" t="n"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
+      <x:c r="I22"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">明細行数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B23" s="7" t="n">
+      <x:c r="A23" t="str">
+        <x:v>明細行数</x:v>
+      </x:c>
+      <x:c r="B23" t="n">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="E23" s="5" t="n"/>
-      <x:c r="G23" s="5" t="n"/>
-      <x:c r="H23" s="5" t="n"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
+      <x:c r="I23"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">支払合計(税込)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B24" s="7" t="n">
+      <x:c r="A24" t="str">
+        <x:v>税込合計</x:v>
+      </x:c>
+      <x:c r="B24" t="n">
         <x:v>49528</x:v>
       </x:c>
-      <x:c r="E24" s="5" t="n"/>
-      <x:c r="G24" s="5" t="n"/>
-      <x:c r="H24" s="5" t="n"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
+      <x:c r="I24"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" t="str">
-        <x:v>税込合計</x:v>
-      </x:c>
-      <x:c r="B25" s="7" t="n">
-        <x:v>49528</x:v>
-      </x:c>
-      <x:c r="E25" s="5" t="n"/>
-      <x:c r="G25" s="5" t="n"/>
-      <x:c r="H25" s="5" t="n"/>
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="E25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Hide payment method from ledger summary
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R63c0fddc2da44fa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="Rdfd8518cab3e4e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="R3591e3cb47564539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R1961727849494429"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R6601469aa2d34525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="Rb830b699946e42a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9532,17 +9532,15 @@
         <x:v>税込合計</x:v>
       </x:c>
       <x:c r="F1" t="str">
-        <x:v>支払方法</x:v>
+        <x:v>読取信頼度</x:v>
       </x:c>
       <x:c r="G1" t="str">
-        <x:v>読取信頼度</x:v>
+        <x:v>備考</x:v>
       </x:c>
       <x:c r="H1" t="str">
-        <x:v>備考</x:v>
-      </x:c>
-      <x:c r="I1" t="str">
         <x:v>画像</x:v>
       </x:c>
+      <x:c r="I1"/>
       <x:c r="J1"/>
       <x:c r="K1"/>
       <x:c r="L1"/>
@@ -9564,17 +9562,15 @@
         <x:v>6923</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>高</x:v>
+        <x:v>税込合計6,923円に統一。消費税等512円を明細に追加。</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>税込合計6,923円に統一。消費税等512円を明細に追加。</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
         <x:v>receipt_images/R20260509-AEON_IMG_8759.JPG</x:v>
       </x:c>
+      <x:c r="I2"/>
       <x:c r="J2"/>
       <x:c r="K2"/>
       <x:c r="L2"/>
@@ -9596,17 +9592,15 @@
         <x:v>1355</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>高</x:v>
+        <x:v>今川焼は50%値引後で実質単価を算出。</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>今川焼は50%値引後で実質単価を算出。</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
         <x:v>receipt_images/R20260512-AEON_IMG_8757.JPG</x:v>
       </x:c>
+      <x:c r="I3"/>
       <x:c r="J3"/>
       <x:c r="K3"/>
       <x:c r="L3"/>
@@ -9628,17 +9622,15 @@
         <x:v>1179</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>高</x:v>
+        <x:v>税込支払額1,179円に訂正。消費税等87円を明細に追加。</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>税込支払額1,179円に訂正。消費税等87円を明細に追加。</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
         <x:v>receipt_images/R20260510-GYOMU_IMG_8757.JPG</x:v>
       </x:c>
+      <x:c r="I4"/>
       <x:c r="J4"/>
       <x:c r="K4"/>
       <x:c r="L4"/>
@@ -9660,17 +9652,15 @@
         <x:v>388</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>JCB</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>中</x:v>
+        <x:v>商品名はレシート画像から読める範囲。内消費税28円。</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>商品名はレシート画像から読める範囲。内消費税28円。</x:v>
-      </x:c>
-      <x:c r="I5" t="str">
         <x:v>receipt_images/R20260512-LETAO_IMG_8760.JPG</x:v>
       </x:c>
+      <x:c r="I5"/>
       <x:c r="J5"/>
       <x:c r="K5"/>
       <x:c r="L5"/>
@@ -9692,17 +9682,15 @@
         <x:v>2201</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>中</x:v>
+        <x:v>領収書。値引は読取可能範囲で反映。税込合計2,201円。</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>領収書。値引は読取可能範囲で反映。税込合計2,201円。</x:v>
-      </x:c>
-      <x:c r="I6" t="str">
         <x:v>receipt_images/R20260512-COOP_IMG_8760.JPG</x:v>
       </x:c>
+      <x:c r="I6"/>
       <x:c r="J6"/>
       <x:c r="K6"/>
       <x:c r="L6"/>
@@ -9724,17 +9712,15 @@
         <x:v>6042</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>高</x:v>
+        <x:v>灯油 41.96L、単価144円。内税10%対象。</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>灯油 41.96L、単価144円。内税10%対象。</x:v>
-      </x:c>
-      <x:c r="I7" t="str">
         <x:v>receipt_images/R20260412-APOLLO_IMG_8761_2.JPG</x:v>
       </x:c>
+      <x:c r="I7"/>
       <x:c r="J7"/>
       <x:c r="K7"/>
       <x:c r="L7"/>
@@ -9756,17 +9742,15 @@
         <x:v>2124</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>中</x:v>
+        <x:v>IMG_8765左。明細合計一致。</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>IMG_8765左。明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I8" t="str">
         <x:v>receipt_images/R20260423-AEON-1917_IMG_8765.JPG</x:v>
       </x:c>
+      <x:c r="I8"/>
       <x:c r="J8"/>
       <x:c r="K8"/>
       <x:c r="L8"/>
@@ -9788,17 +9772,15 @@
         <x:v>220</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>現金</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>高</x:v>
+        <x:v>B5ノート 2個。税込220円に訂正。</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>B5ノート 2個。税込220円に訂正。</x:v>
-      </x:c>
-      <x:c r="I9" t="str">
         <x:v>receipt_images/R20260423-CANDO-1602_IMG_8765.JPG</x:v>
       </x:c>
+      <x:c r="I9"/>
       <x:c r="J9"/>
       <x:c r="K9"/>
       <x:c r="L9"/>
@@ -9820,17 +9802,15 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>高</x:v>
+        <x:v>税込合計535円。</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>税込合計535円。</x:v>
-      </x:c>
-      <x:c r="I10" t="str">
         <x:v>receipt_images/R20260510-SUNDRUG-1326_IMG_8765.JPG</x:v>
       </x:c>
+      <x:c r="I10"/>
       <x:c r="J10"/>
       <x:c r="K10"/>
       <x:c r="L10"/>
@@ -9852,17 +9832,15 @@
         <x:v>1578</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>中</x:v>
+        <x:v>IMG_8765中央右。明細合計一致。</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>IMG_8765中央右。明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I11" t="str">
         <x:v>receipt_images/R20260510-AEON-1911_IMG_8765.JPG</x:v>
       </x:c>
+      <x:c r="I11"/>
       <x:c r="J11"/>
       <x:c r="K11"/>
       <x:c r="L11"/>
@@ -9884,17 +9862,15 @@
         <x:v>2744</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>中</x:v>
+        <x:v>IMG_8765右。明細合計一致。</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>IMG_8765右。明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I12" t="str">
         <x:v>receipt_images/R20260505-AEON-1930_IMG_8765.JPG</x:v>
       </x:c>
+      <x:c r="I12"/>
       <x:c r="J12"/>
       <x:c r="K12"/>
       <x:c r="L12"/>
@@ -9916,17 +9892,15 @@
         <x:v>705</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>低</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>低</x:v>
+        <x:v>IMG_8764左。明細読取に差額あり。</x:v>
       </x:c>
       <x:c r="H13" t="str">
-        <x:v>IMG_8764左。明細読取に差額あり。</x:v>
-      </x:c>
-      <x:c r="I13" t="str">
         <x:v>receipt_images/R20260429-AEON-MAXVALU-1437_IMG_8764_2.JPG</x:v>
       </x:c>
+      <x:c r="I13"/>
       <x:c r="J13"/>
       <x:c r="K13"/>
       <x:c r="L13"/>
@@ -9948,17 +9922,15 @@
         <x:v>555</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>高</x:v>
+        <x:v>明細合計一致。</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I14" t="str">
         <x:v>receipt_images/R20260429-AEON-1746_IMG_8764_2.JPG</x:v>
       </x:c>
+      <x:c r="I14"/>
       <x:c r="J14"/>
       <x:c r="K14"/>
       <x:c r="L14"/>
@@ -9980,17 +9952,15 @@
         <x:v>6000</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>中</x:v>
+        <x:v>8%対象4,181円、10%対象1,350円。明細合計一致。</x:v>
       </x:c>
       <x:c r="H15" t="str">
-        <x:v>8%対象4,181円、10%対象1,350円。明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I15" t="str">
         <x:v>receipt_images/R20260427-AEON-1920_IMG_8764_2.JPG</x:v>
       </x:c>
+      <x:c r="I15"/>
       <x:c r="J15"/>
       <x:c r="K15"/>
       <x:c r="L15"/>
@@ -10012,17 +9982,15 @@
         <x:v>4514</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>高</x:v>
+        <x:v>レギュラーガソリン 28.04L、単価166円、値引140円。</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>レギュラーガソリン 28.04L、単価166円、値引140円。</x:v>
-      </x:c>
-      <x:c r="I16" t="str">
         <x:v>receipt_images/R20260423-APOLLO-1702_IMG_8764_2.JPG</x:v>
       </x:c>
+      <x:c r="I16"/>
       <x:c r="J16"/>
       <x:c r="K16"/>
       <x:c r="L16"/>
@@ -10044,17 +10012,15 @@
         <x:v>4498</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>中</x:v>
+        <x:v>IMG_8763左。明細合計一致。</x:v>
       </x:c>
       <x:c r="H17" t="str">
-        <x:v>IMG_8763左。明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I17" t="str">
         <x:v>receipt_images/R20260504-AEON-1918_IMG_8763_2.JPG</x:v>
       </x:c>
+      <x:c r="I17"/>
       <x:c r="J17"/>
       <x:c r="K17"/>
       <x:c r="L17"/>
@@ -10076,17 +10042,15 @@
         <x:v>3965</x:v>
       </x:c>
       <x:c r="F18" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>中</x:v>
+        <x:v>IMG_8766で再確認。明細合計一致。</x:v>
       </x:c>
       <x:c r="H18" t="str">
-        <x:v>IMG_8766で再確認。明細合計一致。</x:v>
-      </x:c>
-      <x:c r="I18" t="str">
         <x:v>receipt_images/R20260423-GYOMU-1651_IMG_8766.JPG</x:v>
       </x:c>
+      <x:c r="I18"/>
       <x:c r="J18"/>
       <x:c r="K18"/>
       <x:c r="L18"/>
@@ -10108,17 +10072,15 @@
         <x:v>966</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>中</x:v>
+        <x:v>商品名は画像から読める範囲。</x:v>
       </x:c>
       <x:c r="H19" t="str">
-        <x:v>商品名は画像から読める範囲。</x:v>
-      </x:c>
-      <x:c r="I19" t="str">
         <x:v>receipt_images/R20260429-NISHIMATSUYA-1518_IMG_8763_2.JPG</x:v>
       </x:c>
+      <x:c r="I19"/>
       <x:c r="J19"/>
       <x:c r="K19"/>
       <x:c r="L19"/>
@@ -10140,17 +10102,15 @@
         <x:v>3036</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>クレジット</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>高</x:v>
+        <x:v>税込合計3,036円。</x:v>
       </x:c>
       <x:c r="H20" t="str">
-        <x:v>税込合計3,036円。</x:v>
-      </x:c>
-      <x:c r="I20" t="str">
         <x:v>receipt_images/R20260423-DCM-1619_IMG_8763_2.JPG</x:v>
       </x:c>
+      <x:c r="I20"/>
       <x:c r="J20"/>
       <x:c r="K20"/>
       <x:c r="L20"/>
@@ -10165,6 +10125,8 @@
       <x:c r="G21"/>
       <x:c r="H21"/>
       <x:c r="I21"/>
+      <x:c r="J21"/>
+      <x:c r="K21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
@@ -10180,6 +10142,8 @@
       <x:c r="G22"/>
       <x:c r="H22"/>
       <x:c r="I22"/>
+      <x:c r="J22"/>
+      <x:c r="K22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
@@ -10195,6 +10159,8 @@
       <x:c r="G23"/>
       <x:c r="H23"/>
       <x:c r="I23"/>
+      <x:c r="J23"/>
+      <x:c r="K23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
@@ -10210,13 +10176,21 @@
       <x:c r="G24"/>
       <x:c r="H24"/>
       <x:c r="I24"/>
+      <x:c r="J24"/>
+      <x:c r="K24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25"/>
       <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
       <x:c r="E25"/>
+      <x:c r="F25"/>
       <x:c r="G25"/>
       <x:c r="H25"/>
+      <x:c r="I25"/>
+      <x:c r="J25"/>
+      <x:c r="K25"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add household budget summary sections
</commit_message>
<xml_diff>
--- a/shopping_receipt_ledger.xlsx
+++ b/shopping_receipt_ledger.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R1961727849494429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R6601469aa2d34525"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="Rb830b699946e42a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明細" sheetId="1" r:id="R7f409a6956a74c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レシート集計" sheetId="2" r:id="R0ee9269f387e4c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最安値ビュー" sheetId="3" r:id="Ree3c7594ddca4b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家計簿サマリー" sheetId="4" r:id="Rbb17840184354e8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -34,13 +36,58 @@
       <x:b/>
       <x:color rgb="FFFFFF"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="DDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="DDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="DDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="DDEBF7"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -54,7 +101,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
@@ -64,6 +111,26 @@
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -13891,4 +13958,145 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13.5" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="7.119999885559082" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>項目内訳別合計</x:v>
+      </x:c>
+      <x:c r="B1" s="28"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="27" t="str">
+        <x:v>分類</x:v>
+      </x:c>
+      <x:c r="B2" s="27" t="str">
+        <x:v>合計</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>食品系</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:v>27355</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>ガソリン・灯油</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>10556</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>日用品</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>619</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>その他</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>8547</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>税・調整</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
+        <x:v>599</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>未分類・差額</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>1852</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9"/>
+      <x:c r="B9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>月別・年間集計</x:v>
+      </x:c>
+      <x:c r="B10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="25" t="str">
+        <x:v>期間</x:v>
+      </x:c>
+      <x:c r="B11" s="25" t="str">
+        <x:v>税込合計</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="27" t="str">
+        <x:v>2026年4月合計</x:v>
+      </x:c>
+      <x:c r="B12" s="27" t="n">
+        <x:v>28127</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>2026年5月合計</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>21401</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>年間合計</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>49528</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>月平均</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:v>24764</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>レシート1枚平均</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
+        <x:v>2607</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>